<commit_message>
updated bolsdorfer models with new 14C value|
</commit_message>
<xml_diff>
--- a/outputs/radiocarbon_main_experiment_statistics_2025_2026.xlsx
+++ b/outputs/radiocarbon_main_experiment_statistics_2025_2026.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="219">
   <si>
     <t xml:space="preserve">Term</t>
   </si>
@@ -627,6 +627,9 @@
   </si>
   <si>
     <t xml:space="preserve">15_2026_Bulk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15_2026_MAOM</t>
   </si>
   <si>
     <t xml:space="preserve">15_2026_fPOM</t>
@@ -1080,22 +1083,22 @@
         <v>8</v>
       </c>
       <c r="B2" t="n">
-        <v>5721.60935540045</v>
+        <v>5507.87081964821</v>
       </c>
       <c r="C2" t="n">
-        <v>1430.40233885011</v>
+        <v>1376.96770491205</v>
       </c>
       <c r="D2" t="n">
         <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>14.1368686349429</v>
+        <v>13.6251633352567</v>
       </c>
       <c r="F2" t="n">
-        <v>1.59346384410476</v>
+        <v>1.52640615137533</v>
       </c>
       <c r="G2" t="n">
-        <v>0.230265321337811</v>
+        <v>0.249469565642342</v>
       </c>
       <c r="H2" t="s">
         <v>9</v>
@@ -1106,22 +1109,22 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>4836.69387966255</v>
+        <v>5737.53043760482</v>
       </c>
       <c r="C3" t="n">
-        <v>4836.69387966255</v>
+        <v>5737.53043760482</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>99.5643726468669</v>
+        <v>99.7728857080289</v>
       </c>
       <c r="F3" t="n">
-        <v>5.38806223460226</v>
+        <v>6.36020853824058</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0223137002054018</v>
+        <v>0.0132527923409425</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
@@ -1132,22 +1135,22 @@
         <v>12</v>
       </c>
       <c r="B4" t="n">
-        <v>56968.9367764699</v>
+        <v>56291.6428565317</v>
       </c>
       <c r="C4" t="n">
-        <v>18989.6455921566</v>
+        <v>18763.8809521772</v>
       </c>
       <c r="D4" t="n">
         <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>99.1242594303473</v>
+        <v>99.557621492153</v>
       </c>
       <c r="F4" t="n">
-        <v>21.1544072892037</v>
+        <v>20.8002723716073</v>
       </c>
       <c r="G4" t="n">
-        <v>0.000000000113322565401775</v>
+        <v>0.000000000152785246505609</v>
       </c>
       <c r="H4" t="s">
         <v>13</v>
@@ -1158,22 +1161,22 @@
         <v>14</v>
       </c>
       <c r="B5" t="n">
-        <v>1573.19447912695</v>
+        <v>1426.52180672882</v>
       </c>
       <c r="C5" t="n">
-        <v>393.298619781738</v>
+        <v>356.630451682206</v>
       </c>
       <c r="D5" t="n">
         <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>99.4633529334022</v>
+        <v>99.7728860183999</v>
       </c>
       <c r="F5" t="n">
-        <v>0.438133463248045</v>
+        <v>0.395334555250335</v>
       </c>
       <c r="G5" t="n">
-        <v>0.780772246868797</v>
+        <v>0.811563767890017</v>
       </c>
       <c r="H5" t="s">
         <v>9</v>
@@ -1184,22 +1187,22 @@
         <v>15</v>
       </c>
       <c r="B6" t="n">
-        <v>9083.85776170894</v>
+        <v>9660.87142229029</v>
       </c>
       <c r="C6" t="n">
-        <v>756.988146809078</v>
+        <v>805.072618524191</v>
       </c>
       <c r="D6" t="n">
         <v>12</v>
       </c>
       <c r="E6" t="n">
-        <v>98.9935062127986</v>
+        <v>99.5576215200008</v>
       </c>
       <c r="F6" t="n">
-        <v>0.84328248744742</v>
+        <v>0.892444893831157</v>
       </c>
       <c r="G6" t="n">
-        <v>0.606121725495332</v>
+        <v>0.557185999551352</v>
       </c>
       <c r="H6" t="s">
         <v>9</v>
@@ -1210,22 +1213,22 @@
         <v>16</v>
       </c>
       <c r="B7" t="n">
-        <v>2433.8457360122</v>
+        <v>2077.52447337181</v>
       </c>
       <c r="C7" t="n">
-        <v>811.281912004066</v>
+        <v>692.508157790602</v>
       </c>
       <c r="D7" t="n">
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>99.1242595112719</v>
+        <v>99.5576217275459</v>
       </c>
       <c r="F7" t="n">
-        <v>0.903765576330004</v>
+        <v>0.767664127603259</v>
       </c>
       <c r="G7" t="n">
-        <v>0.442221855780301</v>
+        <v>0.514799766918507</v>
       </c>
       <c r="H7" t="s">
         <v>9</v>
@@ -1236,22 +1239,22 @@
         <v>17</v>
       </c>
       <c r="B8" t="n">
-        <v>12858.3333043903</v>
+        <v>12768.5626445319</v>
       </c>
       <c r="C8" t="n">
-        <v>1071.52777536586</v>
+        <v>1064.04688704433</v>
       </c>
       <c r="D8" t="n">
         <v>12</v>
       </c>
       <c r="E8" t="n">
-        <v>98.9935063586225</v>
+        <v>99.5576215453978</v>
       </c>
       <c r="F8" t="n">
-        <v>1.19367867461129</v>
+        <v>1.17952491401385</v>
       </c>
       <c r="G8" t="n">
-        <v>0.298252664391704</v>
+        <v>0.308161899587924</v>
       </c>
       <c r="H8" t="s">
         <v>9</v>
@@ -5984,7 +5987,7 @@
         <v>51</v>
       </c>
       <c r="D99" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E99" t="s">
         <v>38</v>
@@ -5993,25 +5996,25 @@
         <v>50</v>
       </c>
       <c r="G99" t="n">
-        <v>0.433381486831886</v>
+        <v>98.6776308478721</v>
       </c>
       <c r="H99" t="n">
-        <v>23.97444916</v>
+        <v>1.26</v>
       </c>
       <c r="I99" t="n">
-        <v>1.397448421</v>
+        <v>0.1</v>
       </c>
       <c r="J99" t="n">
-        <v>17.1558740914703</v>
+        <v>12.6</v>
       </c>
       <c r="K99" t="n">
-        <v>5.49739810737369</v>
+        <v>65.7850872319148</v>
       </c>
       <c r="L99" t="n">
-        <v>4.32591624617037</v>
+        <v>70.4840220341944</v>
       </c>
       <c r="M99" t="n">
-        <v>-85.49</v>
+        <v>-72.55159767</v>
       </c>
     </row>
     <row r="100">
@@ -6025,7 +6028,7 @@
         <v>51</v>
       </c>
       <c r="D100" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E100" t="s">
         <v>38</v>
@@ -6034,25 +6037,25 @@
         <v>50</v>
       </c>
       <c r="G100" t="n">
-        <v>0.888987665295966</v>
+        <v>0.433381486831886</v>
       </c>
       <c r="H100" t="n">
-        <v>35.5</v>
+        <v>23.97444916</v>
       </c>
       <c r="I100" t="n">
-        <v>2.23</v>
+        <v>1.397448421</v>
       </c>
       <c r="J100" t="n">
-        <v>15.9192825112108</v>
+        <v>17.1558740914703</v>
       </c>
       <c r="K100" t="n">
-        <v>16.6979164645539</v>
+        <v>5.49739810737369</v>
       </c>
       <c r="L100" t="n">
-        <v>14.1603035257857</v>
+        <v>4.32591624617037</v>
       </c>
       <c r="M100" t="n">
-        <v>-40.15</v>
+        <v>-85.49</v>
       </c>
     </row>
     <row r="101">
@@ -6060,40 +6063,40 @@
         <v>203</v>
       </c>
       <c r="B101" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C101" t="s">
         <v>51</v>
       </c>
       <c r="D101" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E101" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F101" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="G101" t="n">
-        <v>100</v>
+        <v>0.888987665295966</v>
       </c>
       <c r="H101" t="n">
-        <v>2.05</v>
+        <v>35.5</v>
       </c>
       <c r="I101" t="n">
-        <v>0.15</v>
+        <v>2.23</v>
       </c>
       <c r="J101" t="n">
-        <v>13.6666666666667</v>
+        <v>15.9192825112108</v>
       </c>
       <c r="K101" t="n">
-        <v>100</v>
+        <v>16.6979164645539</v>
       </c>
       <c r="L101" t="n">
-        <v>100</v>
+        <v>14.1603035257857</v>
       </c>
       <c r="M101" t="n">
-        <v>-79.1</v>
+        <v>-40.15</v>
       </c>
     </row>
     <row r="102">
@@ -6107,7 +6110,7 @@
         <v>51</v>
       </c>
       <c r="D102" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E102" t="s">
         <v>36</v>
@@ -6116,25 +6119,25 @@
         <v>2</v>
       </c>
       <c r="G102" t="n">
-        <v>0.917246245338111</v>
+        <v>100</v>
       </c>
       <c r="H102" t="n">
-        <v>32.9607811</v>
+        <v>2.05</v>
       </c>
       <c r="I102" t="n">
-        <v>1.792199969</v>
+        <v>0.15</v>
       </c>
       <c r="J102" t="n">
-        <v>18.391240748872</v>
+        <v>13.6666666666667</v>
       </c>
       <c r="K102" t="n">
-        <v>14.7478793694568</v>
+        <v>100</v>
       </c>
       <c r="L102" t="n">
-        <v>10.9592579497355</v>
+        <v>100</v>
       </c>
       <c r="M102" t="n">
-        <v>-66.24</v>
+        <v>-79.1</v>
       </c>
     </row>
     <row r="103">
@@ -6148,7 +6151,7 @@
         <v>51</v>
       </c>
       <c r="D103" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E103" t="s">
         <v>36</v>
@@ -6157,25 +6160,25 @@
         <v>2</v>
       </c>
       <c r="G103" t="n">
-        <v>6.24937002318305</v>
+        <v>0.917246245338111</v>
       </c>
       <c r="H103" t="n">
-        <v>16.86</v>
+        <v>32.9607811</v>
       </c>
       <c r="I103" t="n">
-        <v>1.21</v>
+        <v>1.792199969</v>
       </c>
       <c r="J103" t="n">
-        <v>13.9338842975207</v>
+        <v>18.391240748872</v>
       </c>
       <c r="K103" t="n">
-        <v>51.3972578492031</v>
+        <v>14.7478793694568</v>
       </c>
       <c r="L103" t="n">
-        <v>50.4115848536766</v>
+        <v>10.9592579497355</v>
       </c>
       <c r="M103" t="n">
-        <v>-9.11</v>
+        <v>-66.24</v>
       </c>
     </row>
     <row r="104">
@@ -6183,40 +6186,40 @@
         <v>206</v>
       </c>
       <c r="B104" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C104" t="s">
         <v>51</v>
       </c>
       <c r="D104" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E104" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F104" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G104" t="n">
-        <v>100</v>
+        <v>6.24937002318305</v>
       </c>
       <c r="H104" t="n">
-        <v>1.98</v>
+        <v>16.86</v>
       </c>
       <c r="I104" t="n">
-        <v>0.14</v>
+        <v>1.21</v>
       </c>
       <c r="J104" t="n">
-        <v>14.1428571428571</v>
+        <v>13.9338842975207</v>
       </c>
       <c r="K104" t="n">
-        <v>100</v>
+        <v>51.3972578492031</v>
       </c>
       <c r="L104" t="n">
-        <v>100</v>
+        <v>50.4115848536766</v>
       </c>
       <c r="M104" t="n">
-        <v>-77.5</v>
+        <v>-9.11</v>
       </c>
     </row>
     <row r="105">
@@ -6230,7 +6233,7 @@
         <v>51</v>
       </c>
       <c r="D105" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E105" t="s">
         <v>35</v>
@@ -6239,25 +6242,25 @@
         <v>0</v>
       </c>
       <c r="G105" t="n">
-        <v>2.3063099041533</v>
+        <v>100</v>
       </c>
       <c r="H105" t="n">
-        <v>16.71080208</v>
+        <v>1.98</v>
       </c>
       <c r="I105" t="n">
-        <v>1.040011287</v>
+        <v>0.14</v>
       </c>
       <c r="J105" t="n">
-        <v>16.0679045399629</v>
+        <v>14.1428571428571</v>
       </c>
       <c r="K105" t="n">
-        <v>19.4647920926513</v>
+        <v>100</v>
       </c>
       <c r="L105" t="n">
-        <v>17.1327737974237</v>
+        <v>100</v>
       </c>
       <c r="M105" t="n">
-        <v>-91.08</v>
+        <v>-77.5</v>
       </c>
     </row>
     <row r="106">
@@ -6271,7 +6274,7 @@
         <v>51</v>
       </c>
       <c r="D106" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E106" t="s">
         <v>35</v>
@@ -6280,25 +6283,25 @@
         <v>0</v>
       </c>
       <c r="G106" t="n">
-        <v>5.84065495207675</v>
+        <v>2.3063099041533</v>
       </c>
       <c r="H106" t="n">
-        <v>20.16</v>
+        <v>16.71080208</v>
       </c>
       <c r="I106" t="n">
-        <v>1.37</v>
+        <v>1.040011287</v>
       </c>
       <c r="J106" t="n">
-        <v>14.7153284671533</v>
+        <v>16.0679045399629</v>
       </c>
       <c r="K106" t="n">
-        <v>59.4684867847814</v>
+        <v>19.4647920926513</v>
       </c>
       <c r="L106" t="n">
-        <v>57.1549806024653</v>
+        <v>17.1327737974237</v>
       </c>
       <c r="M106" t="n">
-        <v>-25.32</v>
+        <v>-91.08</v>
       </c>
     </row>
     <row r="107">
@@ -6306,40 +6309,40 @@
         <v>209</v>
       </c>
       <c r="B107" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C107" t="s">
         <v>51</v>
       </c>
       <c r="D107" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E107" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F107" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="G107" t="n">
-        <v>100</v>
+        <v>5.84065495207675</v>
       </c>
       <c r="H107" t="n">
-        <v>1.88</v>
+        <v>20.16</v>
       </c>
       <c r="I107" t="n">
-        <v>0.13</v>
+        <v>1.37</v>
       </c>
       <c r="J107" t="n">
-        <v>14.4615384615385</v>
+        <v>14.7153284671533</v>
       </c>
       <c r="K107" t="n">
-        <v>100</v>
+        <v>59.4684867847814</v>
       </c>
       <c r="L107" t="n">
-        <v>100</v>
+        <v>57.1549806024653</v>
       </c>
       <c r="M107" t="n">
-        <v>-124.29</v>
+        <v>-25.32</v>
       </c>
     </row>
     <row r="108">
@@ -6353,7 +6356,7 @@
         <v>51</v>
       </c>
       <c r="D108" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E108" t="s">
         <v>39</v>
@@ -6362,25 +6365,25 @@
         <v>50</v>
       </c>
       <c r="G108" t="n">
-        <v>1.28658732711488</v>
+        <v>100</v>
       </c>
       <c r="H108" t="n">
-        <v>29.57481384</v>
+        <v>1.88</v>
       </c>
       <c r="I108" t="n">
-        <v>1.819944382</v>
+        <v>0.13</v>
       </c>
       <c r="J108" t="n">
-        <v>16.2503943156215</v>
+        <v>14.4615384615385</v>
       </c>
       <c r="K108" t="n">
-        <v>20.2396705788966</v>
+        <v>100</v>
       </c>
       <c r="L108" t="n">
-        <v>18.0116721379624</v>
+        <v>100</v>
       </c>
       <c r="M108" t="n">
-        <v>-60.97</v>
+        <v>-124.29</v>
       </c>
     </row>
     <row r="109">
@@ -6394,7 +6397,7 @@
         <v>51</v>
       </c>
       <c r="D109" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E109" t="s">
         <v>39</v>
@@ -6403,25 +6406,25 @@
         <v>50</v>
       </c>
       <c r="G109" t="n">
-        <v>4.57810657231685</v>
+        <v>1.28658732711488</v>
       </c>
       <c r="H109" t="n">
-        <v>30.46</v>
+        <v>29.57481384</v>
       </c>
       <c r="I109" t="n">
-        <v>1.97</v>
+        <v>1.819944382</v>
       </c>
       <c r="J109" t="n">
-        <v>15.4619289340102</v>
+        <v>16.2503943156215</v>
       </c>
       <c r="K109" t="n">
-        <v>74.1750671238145</v>
+        <v>20.2396705788966</v>
       </c>
       <c r="L109" t="n">
-        <v>69.3759226728015</v>
+        <v>18.0116721379624</v>
       </c>
       <c r="M109" t="n">
-        <v>-37.37</v>
+        <v>-60.97</v>
       </c>
     </row>
     <row r="110">
@@ -6429,40 +6432,40 @@
         <v>212</v>
       </c>
       <c r="B110" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C110" t="s">
         <v>51</v>
       </c>
       <c r="D110" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E110" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F110" t="n">
         <v>50</v>
       </c>
       <c r="G110" t="n">
-        <v>100</v>
+        <v>4.57810657231685</v>
       </c>
       <c r="H110" t="n">
-        <v>2.1</v>
+        <v>30.46</v>
       </c>
       <c r="I110" t="n">
-        <v>0.13</v>
+        <v>1.97</v>
       </c>
       <c r="J110" t="n">
-        <v>16.1538461538462</v>
+        <v>15.4619289340102</v>
       </c>
       <c r="K110" t="n">
-        <v>100</v>
+        <v>74.1750671238145</v>
       </c>
       <c r="L110" t="n">
-        <v>100</v>
+        <v>69.3759226728015</v>
       </c>
       <c r="M110" t="n">
-        <v>-160.41</v>
+        <v>-37.37</v>
       </c>
     </row>
     <row r="111">
@@ -6476,7 +6479,7 @@
         <v>51</v>
       </c>
       <c r="D111" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E111" t="s">
         <v>38</v>
@@ -6485,25 +6488,25 @@
         <v>50</v>
       </c>
       <c r="G111" t="n">
-        <v>0.97498940228909</v>
+        <v>100</v>
       </c>
       <c r="H111" t="n">
-        <v>31.58865166</v>
+        <v>2.1</v>
       </c>
       <c r="I111" t="n">
-        <v>1.999277234</v>
+        <v>0.13</v>
       </c>
       <c r="J111" t="n">
-        <v>15.8000356942993</v>
+        <v>16.1538461538462</v>
       </c>
       <c r="K111" t="n">
-        <v>14.6660002862389</v>
+        <v>100</v>
       </c>
       <c r="L111" t="n">
-        <v>14.9944162722142</v>
+        <v>100</v>
       </c>
       <c r="M111" t="n">
-        <v>-87.61</v>
+        <v>-160.41</v>
       </c>
     </row>
     <row r="112">
@@ -6517,7 +6520,7 @@
         <v>51</v>
       </c>
       <c r="D112" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E112" t="s">
         <v>38</v>
@@ -6526,25 +6529,25 @@
         <v>50</v>
       </c>
       <c r="G112" t="n">
-        <v>4.59940652819018</v>
+        <v>0.97498940228909</v>
       </c>
       <c r="H112" t="n">
-        <v>31.58</v>
+        <v>31.58865166</v>
       </c>
       <c r="I112" t="n">
-        <v>2.08</v>
+        <v>1.999277234</v>
       </c>
       <c r="J112" t="n">
-        <v>15.1826923076923</v>
+        <v>15.8000356942993</v>
       </c>
       <c r="K112" t="n">
-        <v>69.1663134096408</v>
+        <v>14.6660002862389</v>
       </c>
       <c r="L112" t="n">
-        <v>73.5905044510428</v>
+        <v>14.9944162722142</v>
       </c>
       <c r="M112" t="n">
-        <v>-32.21</v>
+        <v>-87.61</v>
       </c>
     </row>
     <row r="113">
@@ -6552,40 +6555,40 @@
         <v>215</v>
       </c>
       <c r="B113" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C113" t="s">
         <v>51</v>
       </c>
       <c r="D113" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E113" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F113" t="n">
         <v>50</v>
       </c>
       <c r="G113" t="n">
-        <v>100</v>
+        <v>4.59940652819018</v>
       </c>
       <c r="H113" t="n">
-        <v>1.91</v>
+        <v>31.58</v>
       </c>
       <c r="I113" t="n">
-        <v>0.13</v>
+        <v>2.08</v>
       </c>
       <c r="J113" t="n">
-        <v>14.6923076923077</v>
+        <v>15.1826923076923</v>
       </c>
       <c r="K113" t="n">
-        <v>100</v>
+        <v>69.1663134096408</v>
       </c>
       <c r="L113" t="n">
-        <v>100</v>
+        <v>73.5905044510428</v>
       </c>
       <c r="M113" t="n">
-        <v>-77.19</v>
+        <v>-32.21</v>
       </c>
     </row>
     <row r="114">
@@ -6599,7 +6602,7 @@
         <v>51</v>
       </c>
       <c r="D114" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E114" t="s">
         <v>37</v>
@@ -6608,25 +6611,25 @@
         <v>50</v>
       </c>
       <c r="G114" t="n">
-        <v>0.961223375204896</v>
+        <v>100</v>
       </c>
       <c r="H114" t="n">
-        <v>25.22785378</v>
+        <v>1.91</v>
       </c>
       <c r="I114" t="n">
-        <v>1.287819147</v>
+        <v>0.13</v>
       </c>
       <c r="J114" t="n">
-        <v>19.5895936465681</v>
+        <v>14.6923076923077</v>
       </c>
       <c r="K114" t="n">
-        <v>12.6961270992603</v>
+        <v>100</v>
       </c>
       <c r="L114" t="n">
-        <v>9.52216820871407</v>
+        <v>100</v>
       </c>
       <c r="M114" t="n">
-        <v>-69.77</v>
+        <v>-77.19</v>
       </c>
     </row>
     <row r="115">
@@ -6640,7 +6643,7 @@
         <v>51</v>
       </c>
       <c r="D115" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E115" t="s">
         <v>37</v>
@@ -6649,24 +6652,65 @@
         <v>50</v>
       </c>
       <c r="G115" t="n">
+        <v>0.961223375204896</v>
+      </c>
+      <c r="H115" t="n">
+        <v>25.22785378</v>
+      </c>
+      <c r="I115" t="n">
+        <v>1.287819147</v>
+      </c>
+      <c r="J115" t="n">
+        <v>19.5895936465681</v>
+      </c>
+      <c r="K115" t="n">
+        <v>12.6961270992603</v>
+      </c>
+      <c r="L115" t="n">
+        <v>9.52216820871407</v>
+      </c>
+      <c r="M115" t="n">
+        <v>-69.77</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s">
+        <v>218</v>
+      </c>
+      <c r="B116" t="s">
+        <v>160</v>
+      </c>
+      <c r="C116" t="s">
+        <v>51</v>
+      </c>
+      <c r="D116" t="s">
+        <v>32</v>
+      </c>
+      <c r="E116" t="s">
+        <v>37</v>
+      </c>
+      <c r="F116" t="n">
+        <v>50</v>
+      </c>
+      <c r="G116" t="n">
         <v>3.24412889131588</v>
       </c>
-      <c r="H115" t="n">
+      <c r="H116" t="n">
         <v>35.01</v>
       </c>
-      <c r="I115" t="n">
+      <c r="I116" t="n">
         <v>2.32</v>
       </c>
-      <c r="J115" t="n">
+      <c r="J116" t="n">
         <v>15.0905172413793</v>
       </c>
-      <c r="K115" t="n">
+      <c r="K116" t="n">
         <v>59.4643730287796</v>
       </c>
-      <c r="L115" t="n">
+      <c r="L116" t="n">
         <v>57.8952232911757</v>
       </c>
-      <c r="M115" t="n">
+      <c r="M116" t="n">
         <v>-24.86</v>
       </c>
     </row>
@@ -6751,25 +6795,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="n">
-        <v>-35.4733333333315</v>
+        <v>-35.4733333333313</v>
       </c>
       <c r="D2" t="n">
-        <v>30.5949910134342</v>
+        <v>30.4686599131131</v>
       </c>
       <c r="E2" t="n">
-        <v>175.328714368379</v>
+        <v>176.276267394514</v>
       </c>
       <c r="F2" t="n">
-        <v>-112.687100486097</v>
+        <v>-112.363968393325</v>
       </c>
       <c r="G2" t="n">
-        <v>41.7404338194337</v>
+        <v>41.4173017266619</v>
       </c>
       <c r="H2" t="n">
-        <v>-1.15944905222411</v>
+        <v>-1.16425643380739</v>
       </c>
       <c r="I2" t="n">
-        <v>0.495699538549563</v>
+        <v>0.491786824910405</v>
       </c>
     </row>
     <row r="3">
@@ -6780,25 +6824,25 @@
         <v>27</v>
       </c>
       <c r="C3" t="n">
-        <v>-49.3666666666647</v>
+        <v>-49.3666666666649</v>
       </c>
       <c r="D3" t="n">
-        <v>30.5949910134343</v>
+        <v>30.468659913113</v>
       </c>
       <c r="E3" t="n">
-        <v>175.328714368376</v>
+        <v>176.276267394512</v>
       </c>
       <c r="F3" t="n">
-        <v>-126.58043381943</v>
+        <v>-126.257301726658</v>
       </c>
       <c r="G3" t="n">
-        <v>27.8471004861006</v>
+        <v>27.523968393328</v>
       </c>
       <c r="H3" t="n">
-        <v>-1.61355388681068</v>
+        <v>-1.6202441068115</v>
       </c>
       <c r="I3" t="n">
-        <v>0.402801079009105</v>
+        <v>0.397190346271034</v>
       </c>
     </row>
     <row r="4">
@@ -6812,22 +6856,22 @@
         <v>-13.406666666665</v>
       </c>
       <c r="D4" t="n">
-        <v>30.5949910134343</v>
+        <v>30.4686599131131</v>
       </c>
       <c r="E4" t="n">
-        <v>175.32955693826</v>
+        <v>176.276267394512</v>
       </c>
       <c r="F4" t="n">
-        <v>-90.6204299542191</v>
+        <v>-90.2973017266582</v>
       </c>
       <c r="G4" t="n">
-        <v>63.807096620889</v>
+        <v>63.4839683933282</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.438198091340447</v>
+        <v>-0.440014976204945</v>
       </c>
       <c r="I4" t="n">
-        <v>0.661782099051624</v>
+        <v>0.660465287826069</v>
       </c>
     </row>
     <row r="5">
@@ -6838,25 +6882,25 @@
         <v>27</v>
       </c>
       <c r="C5" t="n">
-        <v>-50.4866666666647</v>
+        <v>-50.4866666666649</v>
       </c>
       <c r="D5" t="n">
-        <v>30.5949910134342</v>
+        <v>30.4686599131132</v>
       </c>
       <c r="E5" t="n">
-        <v>175.328714368379</v>
+        <v>176.27626739451</v>
       </c>
       <c r="F5" t="n">
-        <v>-127.70043381943</v>
+        <v>-127.377301726658</v>
       </c>
       <c r="G5" t="n">
-        <v>26.7271004861004</v>
+        <v>26.4039683933285</v>
       </c>
       <c r="H5" t="n">
-        <v>-1.6501611863359</v>
+        <v>-1.65700318985596</v>
       </c>
       <c r="I5" t="n">
-        <v>0.402801079009105</v>
+        <v>0.397190346271034</v>
       </c>
     </row>
     <row r="6">
@@ -6867,25 +6911,25 @@
         <v>31</v>
       </c>
       <c r="C6" t="n">
-        <v>6.14333333333317</v>
+        <v>6.14333333333322</v>
       </c>
       <c r="D6" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E6" t="n">
-        <v>175.328714368374</v>
+        <v>176.276267394527</v>
       </c>
       <c r="F6" t="n">
-        <v>-71.0704338194323</v>
+        <v>-70.747301726659</v>
       </c>
       <c r="G6" t="n">
-        <v>83.3571004860987</v>
+        <v>83.0339683933254</v>
       </c>
       <c r="H6" t="n">
-        <v>0.200795395907638</v>
+        <v>0.201627946580261</v>
       </c>
       <c r="I6" t="n">
-        <v>0.918218930973778</v>
+        <v>0.914494111400943</v>
       </c>
     </row>
     <row r="7">
@@ -6899,22 +6943,22 @@
         <v>-47.2866666666668</v>
       </c>
       <c r="D7" t="n">
-        <v>30.5949910134343</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E7" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="F7" t="n">
-        <v>-124.500433819432</v>
+        <v>-124.177301726659</v>
       </c>
       <c r="G7" t="n">
-        <v>29.9271004860986</v>
+        <v>29.6039683933254</v>
       </c>
       <c r="H7" t="n">
-        <v>-1.54556890197821</v>
+        <v>-1.5519772383004</v>
       </c>
       <c r="I7" t="n">
-        <v>0.372035348677523</v>
+        <v>0.367383574351595</v>
       </c>
     </row>
     <row r="8">
@@ -6925,25 +6969,25 @@
         <v>31</v>
       </c>
       <c r="C8" t="n">
-        <v>-66.3100000000001</v>
+        <v>-66.31</v>
       </c>
       <c r="D8" t="n">
-        <v>30.5949910134343</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E8" t="n">
-        <v>175.329556938255</v>
+        <v>176.276267394527</v>
       </c>
       <c r="F8" t="n">
-        <v>-143.523763287554</v>
+        <v>-143.200635059992</v>
       </c>
       <c r="G8" t="n">
-        <v>10.903763287554</v>
+        <v>10.5806350599922</v>
       </c>
       <c r="H8" t="n">
-        <v>-2.1673482424258</v>
+        <v>-2.17633463989213</v>
       </c>
       <c r="I8" t="n">
-        <v>0.126228017352646</v>
+        <v>0.123441846208982</v>
       </c>
     </row>
     <row r="9">
@@ -6957,22 +7001,22 @@
         <v>-22.7000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>30.5949910134343</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E9" t="n">
-        <v>175.328714368372</v>
+        <v>176.276267394527</v>
       </c>
       <c r="F9" t="n">
-        <v>-99.9137671527656</v>
+        <v>-99.5906350599923</v>
       </c>
       <c r="G9" t="n">
-        <v>54.5137671527653</v>
+        <v>54.1906350599921</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.74195151716281</v>
+        <v>-0.74502784384786</v>
       </c>
       <c r="I9" t="n">
-        <v>0.918218930973778</v>
+        <v>0.914494111400943</v>
       </c>
     </row>
     <row r="10">
@@ -6986,19 +7030,19 @@
         <v>11.5233333333332</v>
       </c>
       <c r="D10" t="n">
-        <v>30.5949910134343</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E10" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="F10" t="n">
-        <v>-65.6904338194323</v>
+        <v>-65.3673017266589</v>
       </c>
       <c r="G10" t="n">
-        <v>88.7371004860986</v>
+        <v>88.4139683933253</v>
       </c>
       <c r="H10" t="n">
-        <v>0.376641173984109</v>
+        <v>0.378202827633189</v>
       </c>
       <c r="I10" t="n">
         <v>1</v>
@@ -7015,19 +7059,19 @@
         <v>-3.48333333333343</v>
       </c>
       <c r="D11" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E11" t="n">
-        <v>175.328714368372</v>
+        <v>176.276267394527</v>
       </c>
       <c r="F11" t="n">
-        <v>-80.6971004860989</v>
+        <v>-80.3739683933255</v>
       </c>
       <c r="G11" t="n">
-        <v>73.7304338194321</v>
+        <v>73.4073017266587</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.113853059535265</v>
+        <v>-0.114325124349638</v>
       </c>
       <c r="I11" t="n">
         <v>1</v>
@@ -7041,22 +7085,22 @@
         <v>32</v>
       </c>
       <c r="C12" t="n">
-        <v>-8.95333333333346</v>
+        <v>-8.95333333333344</v>
       </c>
       <c r="D12" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E12" t="n">
-        <v>175.329556938253</v>
+        <v>176.27626739453</v>
       </c>
       <c r="F12" t="n">
-        <v>-86.1670966208877</v>
+        <v>-85.8439683933255</v>
       </c>
       <c r="G12" t="n">
-        <v>68.2604299542208</v>
+        <v>67.9373017266586</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.292640495609299</v>
+        <v>-0.293853860290069</v>
       </c>
       <c r="I12" t="n">
         <v>1</v>
@@ -7070,22 +7114,22 @@
         <v>32</v>
       </c>
       <c r="C13" t="n">
-        <v>3.9533333333332</v>
+        <v>3.95333333333326</v>
       </c>
       <c r="D13" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E13" t="n">
-        <v>175.328714368372</v>
+        <v>176.276267394527</v>
       </c>
       <c r="F13" t="n">
-        <v>-73.2604338194323</v>
+        <v>-72.9373017266589</v>
       </c>
       <c r="G13" t="n">
-        <v>81.1671004860987</v>
+        <v>80.8439683933255</v>
       </c>
       <c r="H13" t="n">
-        <v>0.129215051300302</v>
+        <v>0.129750810984368</v>
       </c>
       <c r="I13" t="n">
         <v>1</v>
@@ -7099,25 +7143,25 @@
         <v>33</v>
       </c>
       <c r="C14" t="n">
-        <v>63.1720680833334</v>
+        <v>63.1720680833333</v>
       </c>
       <c r="D14" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E14" t="n">
-        <v>175.328714368374</v>
+        <v>176.276267394527</v>
       </c>
       <c r="F14" t="n">
-        <v>-14.0416990694321</v>
+        <v>-13.718566976659</v>
       </c>
       <c r="G14" t="n">
-        <v>140.385835236099</v>
+        <v>140.062703143326</v>
       </c>
       <c r="H14" t="n">
-        <v>2.06478465888728</v>
+        <v>2.0733458006844</v>
       </c>
       <c r="I14" t="n">
-        <v>0.161662038120886</v>
+        <v>0.158377873065961</v>
       </c>
     </row>
     <row r="15">
@@ -7128,25 +7172,25 @@
         <v>33</v>
       </c>
       <c r="C15" t="n">
-        <v>54.5983738866668</v>
+        <v>54.5983738866667</v>
       </c>
       <c r="D15" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E15" t="n">
-        <v>175.328714368374</v>
+        <v>176.276267394527</v>
       </c>
       <c r="F15" t="n">
-        <v>-22.6153932660988</v>
+        <v>-22.2922611733256</v>
       </c>
       <c r="G15" t="n">
-        <v>131.812141039432</v>
+        <v>131.489008946659</v>
       </c>
       <c r="H15" t="n">
-        <v>1.78455270219535</v>
+        <v>1.79195192838689</v>
       </c>
       <c r="I15" t="n">
-        <v>0.228189248382278</v>
+        <v>0.224567587535397</v>
       </c>
     </row>
     <row r="16">
@@ -7157,25 +7201,25 @@
         <v>33</v>
       </c>
       <c r="C16" t="n">
-        <v>39.3192749000001</v>
+        <v>39.3192749</v>
       </c>
       <c r="D16" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E16" t="n">
-        <v>175.329556938255</v>
+        <v>176.27626739453</v>
       </c>
       <c r="F16" t="n">
-        <v>-37.894488387554</v>
+        <v>-37.5713601599923</v>
       </c>
       <c r="G16" t="n">
-        <v>116.533038187554</v>
+        <v>116.209909959992</v>
       </c>
       <c r="H16" t="n">
-        <v>1.28515399408795</v>
+        <v>1.29048258151578</v>
       </c>
       <c r="I16" t="n">
-        <v>0.264735291788078</v>
+        <v>0.261542519650103</v>
       </c>
     </row>
     <row r="17">
@@ -7186,25 +7230,25 @@
         <v>33</v>
       </c>
       <c r="C17" t="n">
-        <v>46.2556034400002</v>
+        <v>46.2556034400001</v>
       </c>
       <c r="D17" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E17" t="n">
-        <v>175.328714368374</v>
+        <v>176.276267394527</v>
       </c>
       <c r="F17" t="n">
-        <v>-30.9581637127653</v>
+        <v>-30.6350316199922</v>
       </c>
       <c r="G17" t="n">
-        <v>123.469370592766</v>
+        <v>123.146238499992</v>
       </c>
       <c r="H17" t="n">
-        <v>1.51186850879247</v>
+        <v>1.5181371143958</v>
       </c>
       <c r="I17" t="n">
-        <v>0.264735291788078</v>
+        <v>0.261542519650103</v>
       </c>
     </row>
   </sheetData>
@@ -7288,22 +7332,22 @@
         <v>27</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.190000000000232</v>
+        <v>-0.190000000000211</v>
       </c>
       <c r="D2" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E2" t="n">
-        <v>175.328714368374</v>
+        <v>176.276267394532</v>
       </c>
       <c r="F2" t="n">
-        <v>-77.4037671527659</v>
+        <v>-77.0806350599924</v>
       </c>
       <c r="G2" t="n">
-        <v>77.0237671527654</v>
+        <v>76.7006350599919</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.00621016688374912</v>
+        <v>-0.00623591587362335</v>
       </c>
       <c r="I2" t="n">
         <v>1</v>
@@ -7317,22 +7361,22 @@
         <v>27</v>
       </c>
       <c r="C3" t="n">
-        <v>-5.41333333333353</v>
+        <v>-5.41333333333343</v>
       </c>
       <c r="D3" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E3" t="n">
-        <v>175.328714368374</v>
+        <v>176.276267394534</v>
       </c>
       <c r="F3" t="n">
-        <v>-82.6271004860992</v>
+        <v>-82.3039683933256</v>
       </c>
       <c r="G3" t="n">
-        <v>71.8004338194321</v>
+        <v>71.4773017266587</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.176935281038537</v>
+        <v>-0.177668901381636</v>
       </c>
       <c r="I3" t="n">
         <v>1</v>
@@ -7349,22 +7393,22 @@
         <v>-35.5566666666668</v>
       </c>
       <c r="D4" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E4" t="n">
-        <v>175.329556938255</v>
+        <v>176.276267394534</v>
       </c>
       <c r="F4" t="n">
-        <v>-112.770429954221</v>
+        <v>-112.447301726659</v>
       </c>
       <c r="G4" t="n">
-        <v>41.6570966208875</v>
+        <v>41.3339683933254</v>
       </c>
       <c r="H4" t="n">
-        <v>-1.16217280962932</v>
+        <v>-1.16699148462924</v>
       </c>
       <c r="I4" t="n">
-        <v>0.986979238464011</v>
+        <v>0.979160181082327</v>
       </c>
     </row>
     <row r="5">
@@ -7378,19 +7422,19 @@
         <v>-13.0666666666669</v>
       </c>
       <c r="D5" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E5" t="n">
-        <v>175.328714368374</v>
+        <v>176.276267394534</v>
       </c>
       <c r="F5" t="n">
-        <v>-90.2804338194325</v>
+        <v>-89.957301726659</v>
       </c>
       <c r="G5" t="n">
-        <v>64.1471004860988</v>
+        <v>63.8239683933253</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.427085161127494</v>
+        <v>-0.428855968852225</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
@@ -7407,19 +7451,19 @@
         <v>21.0966666666667</v>
       </c>
       <c r="D6" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E6" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="F6" t="n">
-        <v>-56.1171004860988</v>
+        <v>-55.7939683933255</v>
       </c>
       <c r="G6" t="n">
-        <v>98.3104338194322</v>
+        <v>97.987301726659</v>
       </c>
       <c r="H6" t="n">
-        <v>0.689546424687724</v>
+        <v>0.692405466037167</v>
       </c>
       <c r="I6" t="n">
         <v>1</v>
@@ -7436,19 +7480,19 @@
         <v>15.9966666666667</v>
       </c>
       <c r="D7" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E7" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="F7" t="n">
-        <v>-61.2171004860987</v>
+        <v>-60.8939683933255</v>
       </c>
       <c r="G7" t="n">
-        <v>93.2104338194322</v>
+        <v>92.887301726659</v>
       </c>
       <c r="H7" t="n">
-        <v>0.522852471492558</v>
+        <v>0.525020355745356</v>
       </c>
       <c r="I7" t="n">
         <v>1</v>
@@ -7462,22 +7506,22 @@
         <v>31</v>
       </c>
       <c r="C8" t="n">
-        <v>2.37666666666671</v>
+        <v>2.37666666666672</v>
       </c>
       <c r="D8" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E8" t="n">
-        <v>175.329556938251</v>
+        <v>176.27626739453</v>
       </c>
       <c r="F8" t="n">
-        <v>-74.8370966208875</v>
+        <v>-74.5139683933255</v>
       </c>
       <c r="G8" t="n">
-        <v>79.5904299542209</v>
+        <v>79.267301726659</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0776815611948736</v>
+        <v>0.0780036494366422</v>
       </c>
       <c r="I8" t="n">
         <v>1</v>
@@ -7494,19 +7538,19 @@
         <v>28.3233333333334</v>
       </c>
       <c r="D9" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E9" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="F9" t="n">
-        <v>-48.8904338194322</v>
+        <v>-48.5673017266588</v>
       </c>
       <c r="G9" t="n">
-        <v>105.537100486099</v>
+        <v>105.213968393326</v>
       </c>
       <c r="H9" t="n">
-        <v>0.925750666862314</v>
+        <v>0.929589073300332</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
@@ -7520,22 +7564,22 @@
         <v>32</v>
       </c>
       <c r="C10" t="n">
-        <v>7.48333333333331</v>
+        <v>7.48333333333333</v>
       </c>
       <c r="D10" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E10" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="F10" t="n">
-        <v>-69.7304338194322</v>
+        <v>-69.4073017266589</v>
       </c>
       <c r="G10" t="n">
-        <v>84.6971004860988</v>
+        <v>84.3739683933255</v>
       </c>
       <c r="H10" t="n">
-        <v>0.244593414982451</v>
+        <v>0.245607563794191</v>
       </c>
       <c r="I10" t="n">
         <v>1</v>
@@ -7549,22 +7593,22 @@
         <v>32</v>
       </c>
       <c r="C11" t="n">
-        <v>-1.12333333333334</v>
+        <v>-1.12333333333336</v>
       </c>
       <c r="D11" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E11" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="F11" t="n">
-        <v>-78.3371004860988</v>
+        <v>-78.0139683933256</v>
       </c>
       <c r="G11" t="n">
-        <v>76.0904338194321</v>
+        <v>75.7673017266589</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.0367162498214195</v>
+        <v>-0.036868485077347</v>
       </c>
       <c r="I11" t="n">
         <v>1</v>
@@ -7578,22 +7622,22 @@
         <v>32</v>
       </c>
       <c r="C12" t="n">
-        <v>-5.23666666666669</v>
+        <v>-5.23666666666666</v>
       </c>
       <c r="D12" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E12" t="n">
-        <v>175.329556938253</v>
+        <v>176.27626739453</v>
       </c>
       <c r="F12" t="n">
-        <v>-82.4504299542209</v>
+        <v>-82.1273017266588</v>
       </c>
       <c r="G12" t="n">
-        <v>71.9770966208876</v>
+        <v>71.6539683933255</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.171160915339614</v>
+        <v>-0.171870593639498</v>
       </c>
       <c r="I12" t="n">
         <v>1</v>
@@ -7607,22 +7651,22 @@
         <v>32</v>
       </c>
       <c r="C13" t="n">
-        <v>8.19666666666664</v>
+        <v>8.19666666666668</v>
       </c>
       <c r="D13" t="n">
-        <v>30.5949910134344</v>
+        <v>30.4686599131127</v>
       </c>
       <c r="E13" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="F13" t="n">
-        <v>-69.0171004860989</v>
+        <v>-68.6939683933255</v>
       </c>
       <c r="G13" t="n">
-        <v>85.4104338194321</v>
+        <v>85.0873017266589</v>
       </c>
       <c r="H13" t="n">
-        <v>0.267908778370533</v>
+        <v>0.26901959882847</v>
       </c>
       <c r="I13" t="n">
         <v>1</v>
@@ -7636,22 +7680,22 @@
         <v>33</v>
       </c>
       <c r="C14" t="n">
-        <v>1.81809024322445</v>
+        <v>1.85799047437918</v>
       </c>
       <c r="D14" t="n">
-        <v>37.7930797571309</v>
+        <v>37.6530736656208</v>
       </c>
       <c r="E14" t="n">
-        <v>175.585158321594</v>
+        <v>176.326806165861</v>
       </c>
       <c r="F14" t="n">
-        <v>-93.5603219994799</v>
+        <v>-93.1629312666422</v>
       </c>
       <c r="G14" t="n">
-        <v>97.1965024859288</v>
+        <v>96.8789122154006</v>
       </c>
       <c r="H14" t="n">
-        <v>0.0481064325772871</v>
+        <v>0.0493449881642895</v>
       </c>
       <c r="I14" t="n">
         <v>1</v>
@@ -7665,22 +7709,22 @@
         <v>33</v>
       </c>
       <c r="C15" t="n">
-        <v>-17.6106248636421</v>
+        <v>-17.4777394626452</v>
       </c>
       <c r="D15" t="n">
-        <v>37.793079757131</v>
+        <v>37.6530736656208</v>
       </c>
       <c r="E15" t="n">
-        <v>175.585158321594</v>
+        <v>176.326806165861</v>
       </c>
       <c r="F15" t="n">
-        <v>-112.989037106347</v>
+        <v>-112.498661203667</v>
       </c>
       <c r="G15" t="n">
-        <v>77.7677873790624</v>
+        <v>77.5431822783762</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.4659748551008</v>
+        <v>-0.464178293061988</v>
       </c>
       <c r="I15" t="n">
         <v>1</v>
@@ -7694,22 +7738,22 @@
         <v>33</v>
       </c>
       <c r="C16" t="n">
-        <v>-18.4623153109836</v>
+        <v>-1.28546154788245</v>
       </c>
       <c r="D16" t="n">
-        <v>46.5479535656935</v>
+        <v>37.6530736656208</v>
       </c>
       <c r="E16" t="n">
-        <v>175.620070785726</v>
+        <v>176.326806165861</v>
       </c>
       <c r="F16" t="n">
-        <v>-135.935163587956</v>
+        <v>-96.3063832889039</v>
       </c>
       <c r="G16" t="n">
-        <v>99.0105329659887</v>
+        <v>93.735460193139</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.396630010488594</v>
+        <v>-0.0341396179047169</v>
       </c>
       <c r="I16" t="n">
         <v>1</v>
@@ -7723,22 +7767,22 @@
         <v>33</v>
       </c>
       <c r="C17" t="n">
-        <v>17.6136440063797</v>
+        <v>18.2689945202046</v>
       </c>
       <c r="D17" t="n">
-        <v>37.7930797571309</v>
+        <v>37.6530736656208</v>
       </c>
       <c r="E17" t="n">
-        <v>175.585158321594</v>
+        <v>176.326806165861</v>
       </c>
       <c r="F17" t="n">
-        <v>-77.7647682363247</v>
+        <v>-76.7519272208168</v>
       </c>
       <c r="G17" t="n">
-        <v>112.992056249084</v>
+        <v>113.289916261226</v>
       </c>
       <c r="H17" t="n">
-        <v>0.466054741226964</v>
+        <v>0.485192648080816</v>
       </c>
       <c r="I17" t="n">
         <v>1</v>
@@ -7830,25 +7874,25 @@
         <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>-4.349999999998</v>
+        <v>-4.34999999999806</v>
       </c>
       <c r="E2" t="n">
-        <v>30.3702753200588</v>
+        <v>30.3694702603565</v>
       </c>
       <c r="F2" t="n">
-        <v>152.112477383327</v>
+        <v>152.969980850413</v>
       </c>
       <c r="G2" t="n">
-        <v>-64.3520125164663</v>
+        <v>-64.3477251748001</v>
       </c>
       <c r="H2" t="n">
-        <v>55.6520125164703</v>
+        <v>55.6477251748039</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.143232155591455</v>
+        <v>-0.143235952511046</v>
       </c>
       <c r="J2" t="n">
-        <v>0.886296398954244</v>
+        <v>0.886292343721875</v>
       </c>
     </row>
     <row r="3">
@@ -7862,25 +7906,25 @@
         <v>27</v>
       </c>
       <c r="D3" t="n">
-        <v>30.9333333333332</v>
+        <v>30.9333333333331</v>
       </c>
       <c r="E3" t="n">
-        <v>30.3702753200585</v>
+        <v>30.3694702603562</v>
       </c>
       <c r="F3" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G3" t="n">
-        <v>-29.0686791831345</v>
+        <v>-29.0643918414683</v>
       </c>
       <c r="H3" t="n">
-        <v>90.935345849801</v>
+        <v>90.9310585081344</v>
       </c>
       <c r="I3" t="n">
-        <v>1.01853977309527</v>
+        <v>1.01856677341234</v>
       </c>
       <c r="J3" t="n">
-        <v>0.310038759622848</v>
+        <v>0.31001692645794</v>
       </c>
     </row>
     <row r="4">
@@ -7894,25 +7938,25 @@
         <v>27</v>
       </c>
       <c r="D4" t="n">
-        <v>39.6033333333332</v>
+        <v>39.6033333333335</v>
       </c>
       <c r="E4" t="n">
-        <v>30.3702753200585</v>
+        <v>30.3694702603561</v>
       </c>
       <c r="F4" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G4" t="n">
-        <v>-20.3986791831346</v>
+        <v>-20.3943918414678</v>
       </c>
       <c r="H4" t="n">
-        <v>99.605345849801</v>
+        <v>99.6010585081347</v>
       </c>
       <c r="I4" t="n">
-        <v>1.30401627630872</v>
+        <v>1.30405084427933</v>
       </c>
       <c r="J4" t="n">
-        <v>0.194197895092006</v>
+        <v>0.194175115053758</v>
       </c>
     </row>
     <row r="5">
@@ -7929,22 +7973,22 @@
         <v>-26.4999999999998</v>
       </c>
       <c r="E5" t="n">
-        <v>30.3702753200586</v>
+        <v>30.3694702603561</v>
       </c>
       <c r="F5" t="n">
-        <v>152.112477383304</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G5" t="n">
-        <v>-86.5020125164676</v>
+        <v>-86.4977251748011</v>
       </c>
       <c r="H5" t="n">
-        <v>33.5020125164681</v>
+        <v>33.4977251748015</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.872563706477082</v>
+        <v>-0.872586837136653</v>
       </c>
       <c r="J5" t="n">
-        <v>0.384276198287212</v>
+        <v>0.384255928016126</v>
       </c>
     </row>
     <row r="6">
@@ -7958,25 +8002,25 @@
         <v>27</v>
       </c>
       <c r="D6" t="n">
-        <v>33.0699999999999</v>
+        <v>33.07</v>
       </c>
       <c r="E6" t="n">
-        <v>30.3702753200585</v>
+        <v>30.3694702603562</v>
       </c>
       <c r="F6" t="n">
-        <v>152.112477383304</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G6" t="n">
-        <v>-26.9320125164679</v>
+        <v>-26.9277251748014</v>
       </c>
       <c r="H6" t="n">
-        <v>93.0720125164677</v>
+        <v>93.0677251748013</v>
       </c>
       <c r="I6" t="n">
-        <v>1.08889365181876</v>
+        <v>1.0889225171362</v>
       </c>
       <c r="J6" t="n">
-        <v>0.277922929598306</v>
+        <v>0.277900602835725</v>
       </c>
     </row>
     <row r="7">
@@ -7993,22 +8037,22 @@
         <v>-11.5600000000002</v>
       </c>
       <c r="E7" t="n">
-        <v>30.3702753200586</v>
+        <v>30.3694702603561</v>
       </c>
       <c r="F7" t="n">
-        <v>152.112477383309</v>
+        <v>152.96998085039</v>
       </c>
       <c r="G7" t="n">
-        <v>-71.5620125164681</v>
+        <v>-71.5577251748014</v>
       </c>
       <c r="H7" t="n">
-        <v>48.4420125164677</v>
+        <v>48.437725174801</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.380635337617936</v>
+        <v>-0.38064542782264</v>
       </c>
       <c r="J7" t="n">
-        <v>0.704004887752</v>
+        <v>0.703994441018627</v>
       </c>
     </row>
     <row r="8">
@@ -8025,22 +8069,22 @@
         <v>3.39333333333334</v>
       </c>
       <c r="E8" t="n">
-        <v>30.3702753200586</v>
+        <v>30.3694702603562</v>
       </c>
       <c r="F8" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G8" t="n">
-        <v>-56.6086791831345</v>
+        <v>-56.604391841468</v>
       </c>
       <c r="H8" t="n">
-        <v>63.3953458498012</v>
+        <v>63.3910585081347</v>
       </c>
       <c r="I8" t="n">
-        <v>0.111732057005494</v>
+        <v>0.111735018893726</v>
       </c>
       <c r="J8" t="n">
-        <v>0.911183162214163</v>
+        <v>0.911179992569331</v>
       </c>
     </row>
     <row r="9">
@@ -8057,22 +8101,22 @@
         <v>51.7233333333334</v>
       </c>
       <c r="E9" t="n">
-        <v>30.3702753200586</v>
+        <v>30.3694702603562</v>
       </c>
       <c r="F9" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G9" t="n">
-        <v>-8.2786791831345</v>
+        <v>-8.27439184146793</v>
       </c>
       <c r="H9" t="n">
-        <v>111.725345849801</v>
+        <v>111.721058508135</v>
       </c>
       <c r="I9" t="n">
-        <v>1.70309069602579</v>
+        <v>1.70313584299994</v>
       </c>
       <c r="J9" t="n">
-        <v>0.090593438701771</v>
+        <v>0.0905735242442888</v>
       </c>
     </row>
     <row r="10">
@@ -8086,25 +8130,25 @@
         <v>31</v>
       </c>
       <c r="D10" t="n">
-        <v>57.1266666666667</v>
+        <v>57.1266666666666</v>
       </c>
       <c r="E10" t="n">
-        <v>30.3702753200586</v>
+        <v>30.3694702603561</v>
       </c>
       <c r="F10" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G10" t="n">
-        <v>-2.87534584980122</v>
+        <v>-2.87105850813468</v>
       </c>
       <c r="H10" t="n">
-        <v>117.128679183135</v>
+        <v>117.124391841468</v>
       </c>
       <c r="I10" t="n">
-        <v>1.88100588699426</v>
+        <v>1.88105575029535</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0618823031396273</v>
+        <v>0.0618647441026004</v>
       </c>
     </row>
     <row r="11">
@@ -8121,22 +8165,22 @@
         <v>39.4633333333333</v>
       </c>
       <c r="E11" t="n">
-        <v>30.3702753200586</v>
+        <v>30.3694702603562</v>
       </c>
       <c r="F11" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G11" t="n">
-        <v>-20.5386791831345</v>
+        <v>-20.534391841468</v>
       </c>
       <c r="H11" t="n">
-        <v>99.4653458498012</v>
+        <v>99.4610585081346</v>
       </c>
       <c r="I11" t="n">
-        <v>1.29940650578393</v>
+        <v>1.29944095155483</v>
       </c>
       <c r="J11" t="n">
-        <v>0.195770388786163</v>
+        <v>0.195747602172434</v>
       </c>
     </row>
     <row r="12">
@@ -8153,22 +8197,22 @@
         <v>6.96666666666656</v>
       </c>
       <c r="E12" t="n">
-        <v>30.3702753200586</v>
+        <v>30.3694702603561</v>
       </c>
       <c r="F12" t="n">
-        <v>152.112477383309</v>
+        <v>152.96998085039</v>
       </c>
       <c r="G12" t="n">
-        <v>-53.0353458498013</v>
+        <v>-53.0310585081346</v>
       </c>
       <c r="H12" t="n">
-        <v>66.9686791831345</v>
+        <v>66.9643918414677</v>
       </c>
       <c r="I12" t="n">
-        <v>0.229390961828564</v>
+        <v>0.229397042718943</v>
       </c>
       <c r="J12" t="n">
-        <v>0.818873210911907</v>
+        <v>0.818866767653136</v>
       </c>
     </row>
     <row r="13">
@@ -8182,25 +8226,25 @@
         <v>32</v>
       </c>
       <c r="D13" t="n">
-        <v>2.92666666666671</v>
+        <v>2.92666666666667</v>
       </c>
       <c r="E13" t="n">
-        <v>30.3702753200586</v>
+        <v>30.3694702603561</v>
       </c>
       <c r="F13" t="n">
-        <v>152.112477383307</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G13" t="n">
-        <v>-57.0753458498012</v>
+        <v>-57.0710585081346</v>
       </c>
       <c r="H13" t="n">
-        <v>62.9286791831346</v>
+        <v>62.9243918414679</v>
       </c>
       <c r="I13" t="n">
-        <v>0.0963661552562132</v>
+        <v>0.096368709812074</v>
       </c>
       <c r="J13" t="n">
-        <v>0.923356616803089</v>
+        <v>0.923353880915312</v>
       </c>
     </row>
     <row r="14">
@@ -8217,22 +8261,22 @@
         <v>9.32666666666664</v>
       </c>
       <c r="E14" t="n">
-        <v>30.3702753200586</v>
+        <v>30.3694702603561</v>
       </c>
       <c r="F14" t="n">
-        <v>152.112477383307</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G14" t="n">
-        <v>-50.6753458498012</v>
+        <v>-50.6710585081346</v>
       </c>
       <c r="H14" t="n">
-        <v>69.3286791831345</v>
+        <v>69.3243918414679</v>
       </c>
       <c r="I14" t="n">
-        <v>0.307098522103508</v>
+        <v>0.30710666293187</v>
       </c>
       <c r="J14" t="n">
-        <v>0.759188400007004</v>
+        <v>0.759179863299396</v>
       </c>
     </row>
     <row r="15">
@@ -8249,22 +8293,22 @@
         <v>10.6833333333333</v>
       </c>
       <c r="E15" t="n">
-        <v>30.3702753200586</v>
+        <v>30.3694702603561</v>
       </c>
       <c r="F15" t="n">
-        <v>152.112477383307</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G15" t="n">
-        <v>-49.3186791831346</v>
+        <v>-49.3143918414679</v>
       </c>
       <c r="H15" t="n">
-        <v>70.6853458498012</v>
+        <v>70.6810585081346</v>
       </c>
       <c r="I15" t="n">
-        <v>0.351769393617493</v>
+        <v>0.351778718619245</v>
       </c>
       <c r="J15" t="n">
-        <v>0.725498038768105</v>
+        <v>0.725488332459841</v>
       </c>
     </row>
     <row r="16">
@@ -8281,22 +8325,22 @@
         <v>11.21</v>
       </c>
       <c r="E16" t="n">
-        <v>30.3702753200586</v>
+        <v>30.3694702603561</v>
       </c>
       <c r="F16" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G16" t="n">
-        <v>-48.7920125164679</v>
+        <v>-48.7877251748013</v>
       </c>
       <c r="H16" t="n">
-        <v>71.2120125164679</v>
+        <v>71.2077251748013</v>
       </c>
       <c r="I16" t="n">
-        <v>0.369110911305969</v>
+        <v>0.369120696011394</v>
       </c>
       <c r="J16" t="n">
-        <v>0.712558340003232</v>
+        <v>0.712548187345262</v>
       </c>
     </row>
     <row r="17">
@@ -8310,25 +8354,25 @@
         <v>33</v>
       </c>
       <c r="D17" t="n">
-        <v>46.4959952105333</v>
+        <v>46.6236293626262</v>
       </c>
       <c r="E17" t="n">
-        <v>34.1831146068425</v>
+        <v>34.1615585662969</v>
       </c>
       <c r="F17" t="n">
-        <v>159.169822953763</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G17" t="n">
-        <v>-21.0149743246288</v>
+        <v>-20.8409989867154</v>
       </c>
       <c r="H17" t="n">
-        <v>114.006964745695</v>
+        <v>114.088257711968</v>
       </c>
       <c r="I17" t="n">
-        <v>1.36020359014407</v>
+        <v>1.3647980747759</v>
       </c>
       <c r="J17" t="n">
-        <v>0.175688808767098</v>
+        <v>0.174228693544156</v>
       </c>
     </row>
     <row r="18">
@@ -8342,25 +8386,25 @@
         <v>33</v>
       </c>
       <c r="D18" t="n">
-        <v>-14.8579826295756</v>
+        <v>-14.6904482463279</v>
       </c>
       <c r="E18" t="n">
-        <v>34.1831146068425</v>
+        <v>34.1615585662968</v>
       </c>
       <c r="F18" t="n">
-        <v>159.169822953761</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G18" t="n">
-        <v>-82.3689521647378</v>
+        <v>-82.1550765956696</v>
       </c>
       <c r="H18" t="n">
-        <v>52.6529869055865</v>
+        <v>52.7741801030137</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.434658538300705</v>
+        <v>-0.430028630509301</v>
       </c>
       <c r="J18" t="n">
-        <v>0.664399000871374</v>
+        <v>0.667752213487498</v>
       </c>
     </row>
     <row r="19">
@@ -8374,25 +8418,25 @@
         <v>33</v>
       </c>
       <c r="D19" t="n">
-        <v>-25.7130035397755</v>
+        <v>-25.4524839866856</v>
       </c>
       <c r="E19" t="n">
-        <v>34.1831146068425</v>
+        <v>34.1615585662968</v>
       </c>
       <c r="F19" t="n">
-        <v>159.16982295376</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G19" t="n">
-        <v>-93.2239730749376</v>
+        <v>-92.9171123360273</v>
       </c>
       <c r="H19" t="n">
-        <v>41.7979659953866</v>
+        <v>42.012144362656</v>
       </c>
       <c r="I19" t="n">
-        <v>-0.752213595382222</v>
+        <v>-0.745062141625955</v>
       </c>
       <c r="J19" t="n">
-        <v>0.453033552577873</v>
+        <v>0.45732487622831</v>
       </c>
     </row>
     <row r="20">
@@ -8406,25 +8450,25 @@
         <v>33</v>
       </c>
       <c r="D20" t="n">
-        <v>-11.2855950004504</v>
+        <v>6.01889291474377</v>
       </c>
       <c r="E20" t="n">
-        <v>43.6678420333502</v>
+        <v>34.1615585662968</v>
       </c>
       <c r="F20" t="n">
-        <v>167.880320952656</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G20" t="n">
-        <v>-97.4944479281164</v>
+        <v>-61.4457354345979</v>
       </c>
       <c r="H20" t="n">
-        <v>74.9232579272155</v>
+        <v>73.4835212640854</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.258441784043996</v>
+        <v>0.176189060667797</v>
       </c>
       <c r="J20" t="n">
-        <v>0.796382547677632</v>
+        <v>0.860367749144128</v>
       </c>
     </row>
     <row r="21">
@@ -8438,25 +8482,25 @@
         <v>33</v>
       </c>
       <c r="D21" t="n">
-        <v>17.8540357769128</v>
+        <v>18.6370204428308</v>
       </c>
       <c r="E21" t="n">
-        <v>34.1831146068425</v>
+        <v>34.1615585662969</v>
       </c>
       <c r="F21" t="n">
-        <v>159.16982295376</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G21" t="n">
-        <v>-49.6569337582493</v>
+        <v>-48.8276079065109</v>
       </c>
       <c r="H21" t="n">
-        <v>85.3650053120749</v>
+        <v>86.1016487921725</v>
       </c>
       <c r="I21" t="n">
-        <v>0.522305705090401</v>
+        <v>0.545555332513947</v>
       </c>
       <c r="J21" t="n">
-        <v>0.602183659883453</v>
+        <v>0.586129796544483</v>
       </c>
     </row>
   </sheetData>
@@ -8545,22 +8589,22 @@
         <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>35.2833333333312</v>
+        <v>35.2833333333311</v>
       </c>
       <c r="E2" t="n">
-        <v>42.9500552506319</v>
+        <v>42.9489167242823</v>
       </c>
       <c r="F2" t="n">
-        <v>152.11247738332</v>
+        <v>152.969980850398</v>
       </c>
       <c r="G2" t="n">
-        <v>-87.0624553018245</v>
+        <v>-87.0490787172946</v>
       </c>
       <c r="H2" t="n">
-        <v>157.629121968487</v>
+        <v>157.615745383957</v>
       </c>
       <c r="I2" t="n">
-        <v>0.821496808966553</v>
+        <v>0.82151858590144</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>
@@ -8577,22 +8621,22 @@
         <v>27</v>
       </c>
       <c r="D3" t="n">
-        <v>43.9533333333312</v>
+        <v>43.9533333333315</v>
       </c>
       <c r="E3" t="n">
-        <v>42.9500552506319</v>
+        <v>42.9489167242823</v>
       </c>
       <c r="F3" t="n">
-        <v>152.112477383317</v>
+        <v>152.969980850401</v>
       </c>
       <c r="G3" t="n">
-        <v>-78.3924553018247</v>
+        <v>-78.379078717294</v>
       </c>
       <c r="H3" t="n">
-        <v>166.299121968487</v>
+        <v>166.285745383957</v>
       </c>
       <c r="I3" t="n">
-        <v>1.0233591802582</v>
+        <v>1.02338630833223</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
@@ -8609,22 +8653,22 @@
         <v>27</v>
       </c>
       <c r="D4" t="n">
-        <v>8.66999999999999</v>
+        <v>8.67000000000039</v>
       </c>
       <c r="E4" t="n">
-        <v>42.9500552506317</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F4" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850393</v>
       </c>
       <c r="G4" t="n">
-        <v>-113.675788635155</v>
+        <v>-113.662412050625</v>
       </c>
       <c r="H4" t="n">
-        <v>131.015788635155</v>
+        <v>131.002412050625</v>
       </c>
       <c r="I4" t="n">
-        <v>0.201862371291652</v>
+        <v>0.201867722430788</v>
       </c>
       <c r="J4" t="n">
         <v>1</v>
@@ -8644,19 +8688,19 @@
         <v>-22.1500000000018</v>
       </c>
       <c r="E5" t="n">
-        <v>42.9500552506319</v>
+        <v>42.9489167242823</v>
       </c>
       <c r="F5" t="n">
-        <v>152.11247738332</v>
+        <v>152.969980850396</v>
       </c>
       <c r="G5" t="n">
-        <v>-144.495788635158</v>
+        <v>-144.482412050627</v>
       </c>
       <c r="H5" t="n">
-        <v>100.195788635154</v>
+        <v>100.182412050624</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.515715285364525</v>
+        <v>-0.515728956383169</v>
       </c>
       <c r="J5" t="n">
         <v>1</v>
@@ -8673,22 +8717,22 @@
         <v>27</v>
       </c>
       <c r="D6" t="n">
-        <v>-57.433333333333</v>
+        <v>-57.4333333333329</v>
       </c>
       <c r="E6" t="n">
-        <v>42.9500552506317</v>
+        <v>42.9489167242821</v>
       </c>
       <c r="F6" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G6" t="n">
-        <v>-179.779121968488</v>
+        <v>-179.765745383958</v>
       </c>
       <c r="H6" t="n">
-        <v>64.9124553018224</v>
+        <v>64.8990787172921</v>
       </c>
       <c r="I6" t="n">
-        <v>-1.33721209433108</v>
+        <v>-1.33724754228462</v>
       </c>
       <c r="J6" t="n">
         <v>1</v>
@@ -8705,22 +8749,22 @@
         <v>27</v>
       </c>
       <c r="D7" t="n">
-        <v>-66.103333333333</v>
+        <v>-66.1033333333333</v>
       </c>
       <c r="E7" t="n">
-        <v>42.9500552506317</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F7" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850393</v>
       </c>
       <c r="G7" t="n">
-        <v>-188.449121968488</v>
+        <v>-188.435745383958</v>
       </c>
       <c r="H7" t="n">
-        <v>56.2424553018225</v>
+        <v>56.2290787172917</v>
       </c>
       <c r="I7" t="n">
-        <v>-1.53907446562274</v>
+        <v>-1.53911526471541</v>
       </c>
       <c r="J7" t="n">
         <v>1</v>
@@ -8737,22 +8781,22 @@
         <v>27</v>
       </c>
       <c r="D8" t="n">
-        <v>37.4199999999979</v>
+        <v>37.419999999998</v>
       </c>
       <c r="E8" t="n">
-        <v>42.9500552506319</v>
+        <v>42.9489167242823</v>
       </c>
       <c r="F8" t="n">
-        <v>152.112477383314</v>
+        <v>152.969980850396</v>
       </c>
       <c r="G8" t="n">
-        <v>-84.9257886351579</v>
+        <v>-84.9124120506278</v>
       </c>
       <c r="H8" t="n">
-        <v>159.765788635154</v>
+        <v>159.752412050624</v>
       </c>
       <c r="I8" t="n">
-        <v>0.871244513694714</v>
+        <v>0.871267609384001</v>
       </c>
       <c r="J8" t="n">
         <v>1</v>
@@ -8769,22 +8813,22 @@
         <v>27</v>
       </c>
       <c r="D9" t="n">
-        <v>2.13666666666663</v>
+        <v>2.13666666666688</v>
       </c>
       <c r="E9" t="n">
-        <v>42.9500552506317</v>
+        <v>42.9489167242821</v>
       </c>
       <c r="F9" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G9" t="n">
-        <v>-120.209121968489</v>
+        <v>-120.195745383958</v>
       </c>
       <c r="H9" t="n">
-        <v>124.482455301822</v>
+        <v>124.469078717292</v>
       </c>
       <c r="I9" t="n">
-        <v>0.049747704728161</v>
+        <v>0.0497490234825614</v>
       </c>
       <c r="J9" t="n">
         <v>1</v>
@@ -8801,22 +8845,22 @@
         <v>27</v>
       </c>
       <c r="D10" t="n">
-        <v>-6.53333333333336</v>
+        <v>-6.5333333333335</v>
       </c>
       <c r="E10" t="n">
-        <v>42.9500552506317</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F10" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850393</v>
       </c>
       <c r="G10" t="n">
-        <v>-128.879121968489</v>
+        <v>-128.865745383958</v>
       </c>
       <c r="H10" t="n">
-        <v>115.812455301822</v>
+        <v>115.799078717291</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.152114666563491</v>
+        <v>-0.152118698948226</v>
       </c>
       <c r="J10" t="n">
         <v>1</v>
@@ -8833,22 +8877,22 @@
         <v>27</v>
       </c>
       <c r="D11" t="n">
-        <v>59.5699999999996</v>
+        <v>59.5699999999998</v>
       </c>
       <c r="E11" t="n">
-        <v>42.9500552506317</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F11" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G11" t="n">
-        <v>-62.7757886351558</v>
+        <v>-62.7624120506252</v>
       </c>
       <c r="H11" t="n">
-        <v>181.915788635155</v>
+        <v>181.902412050625</v>
       </c>
       <c r="I11" t="n">
-        <v>1.38695979905925</v>
+        <v>1.38699656576718</v>
       </c>
       <c r="J11" t="n">
         <v>1</v>
@@ -8868,19 +8912,19 @@
         <v>14.9533333333335</v>
       </c>
       <c r="E12" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F12" t="n">
-        <v>152.112477383307</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G12" t="n">
-        <v>-107.392455301822</v>
+        <v>-107.379078717291</v>
       </c>
       <c r="H12" t="n">
-        <v>137.299121968489</v>
+        <v>137.285745383958</v>
       </c>
       <c r="I12" t="n">
-        <v>0.348156323573381</v>
+        <v>0.348165552796803</v>
       </c>
       <c r="J12" t="n">
         <v>1</v>
@@ -8900,19 +8944,19 @@
         <v>63.2833333333336</v>
       </c>
       <c r="E13" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F13" t="n">
-        <v>152.112477383307</v>
+        <v>152.96998085039</v>
       </c>
       <c r="G13" t="n">
-        <v>-59.062455301822</v>
+        <v>-59.0490787172914</v>
       </c>
       <c r="H13" t="n">
-        <v>185.629121968489</v>
+        <v>185.615745383958</v>
       </c>
       <c r="I13" t="n">
-        <v>1.47341680852442</v>
+        <v>1.47345586710817</v>
       </c>
       <c r="J13" t="n">
         <v>1</v>
@@ -8932,19 +8976,19 @@
         <v>48.33</v>
       </c>
       <c r="E14" t="n">
-        <v>42.9500552506317</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F14" t="n">
-        <v>152.112477383307</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G14" t="n">
-        <v>-74.0157886351556</v>
+        <v>-74.0024120506249</v>
       </c>
       <c r="H14" t="n">
-        <v>170.675788635156</v>
+        <v>170.662412050625</v>
       </c>
       <c r="I14" t="n">
-        <v>1.12526048495104</v>
+        <v>1.12529031431137</v>
       </c>
       <c r="J14" t="n">
         <v>1</v>
@@ -8961,22 +9005,22 @@
         <v>31</v>
       </c>
       <c r="D15" t="n">
-        <v>68.6866666666669</v>
+        <v>68.6866666666668</v>
       </c>
       <c r="E15" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F15" t="n">
-        <v>152.112477383307</v>
+        <v>152.96998085039</v>
       </c>
       <c r="G15" t="n">
-        <v>-53.6591219684888</v>
+        <v>-53.6457453839582</v>
       </c>
       <c r="H15" t="n">
-        <v>191.032455301822</v>
+        <v>191.019078717292</v>
       </c>
       <c r="I15" t="n">
-        <v>1.59922184653433</v>
+        <v>1.59926424006484</v>
       </c>
       <c r="J15" t="n">
         <v>1</v>
@@ -8993,22 +9037,22 @@
         <v>31</v>
       </c>
       <c r="D16" t="n">
-        <v>53.7333333333333</v>
+        <v>53.7333333333332</v>
       </c>
       <c r="E16" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F16" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G16" t="n">
-        <v>-68.6124553018223</v>
+        <v>-68.5990787172917</v>
       </c>
       <c r="H16" t="n">
-        <v>176.079121968489</v>
+        <v>176.065745383958</v>
       </c>
       <c r="I16" t="n">
-        <v>1.25106552296095</v>
+        <v>1.25109868726803</v>
       </c>
       <c r="J16" t="n">
         <v>1</v>
@@ -9025,22 +9069,22 @@
         <v>31</v>
       </c>
       <c r="D17" t="n">
-        <v>5.4033333333333</v>
+        <v>5.4033333333332</v>
       </c>
       <c r="E17" t="n">
-        <v>42.9500552506317</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F17" t="n">
-        <v>152.112477383307</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G17" t="n">
-        <v>-116.942455301822</v>
+        <v>-116.929078717292</v>
       </c>
       <c r="H17" t="n">
-        <v>127.749121968489</v>
+        <v>127.735745383958</v>
       </c>
       <c r="I17" t="n">
-        <v>0.125805038009906</v>
+        <v>0.125808372956664</v>
       </c>
       <c r="J17" t="n">
         <v>1</v>
@@ -9060,19 +9104,19 @@
         <v>51.0233333333335</v>
       </c>
       <c r="E18" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F18" t="n">
-        <v>152.112477383307</v>
+        <v>152.96998085039</v>
       </c>
       <c r="G18" t="n">
-        <v>-71.3224553018221</v>
+        <v>-71.3090787172914</v>
       </c>
       <c r="H18" t="n">
-        <v>173.369121968489</v>
+        <v>173.355745383958</v>
       </c>
       <c r="I18" t="n">
-        <v>1.18796898014661</v>
+        <v>1.18800047183696</v>
       </c>
       <c r="J18" t="n">
         <v>1</v>
@@ -9092,19 +9136,19 @@
         <v>36.07</v>
       </c>
       <c r="E19" t="n">
-        <v>42.9500552506317</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F19" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G19" t="n">
-        <v>-86.2757886351556</v>
+        <v>-86.262412050625</v>
       </c>
       <c r="H19" t="n">
-        <v>158.415788635156</v>
+        <v>158.402412050625</v>
       </c>
       <c r="I19" t="n">
-        <v>0.839812656573228</v>
+        <v>0.83983491904016</v>
       </c>
       <c r="J19" t="n">
         <v>1</v>
@@ -9121,22 +9165,22 @@
         <v>31</v>
       </c>
       <c r="D20" t="n">
-        <v>-12.26</v>
+        <v>-12.2600000000001</v>
       </c>
       <c r="E20" t="n">
-        <v>42.9500552506317</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F20" t="n">
-        <v>152.112477383307</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G20" t="n">
-        <v>-134.605788635156</v>
+        <v>-134.592412050625</v>
       </c>
       <c r="H20" t="n">
-        <v>110.085788635156</v>
+        <v>110.072412050625</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.285447828377816</v>
+        <v>-0.285455395271207</v>
       </c>
       <c r="J20" t="n">
         <v>1</v>
@@ -9156,19 +9200,19 @@
         <v>-17.6633333333333</v>
       </c>
       <c r="E21" t="n">
-        <v>42.9500552506317</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F21" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G21" t="n">
-        <v>-140.009121968489</v>
+        <v>-139.995745383958</v>
       </c>
       <c r="H21" t="n">
-        <v>104.682455301822</v>
+        <v>104.669078717292</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.411252866387722</v>
+        <v>-0.411263768227871</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
@@ -9185,22 +9229,22 @@
         <v>32</v>
       </c>
       <c r="D22" t="n">
-        <v>-4.03999999999985</v>
+        <v>-4.03999999999989</v>
       </c>
       <c r="E22" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F22" t="n">
-        <v>152.11247738331</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G22" t="n">
-        <v>-126.385788635155</v>
+        <v>-126.372412050625</v>
       </c>
       <c r="H22" t="n">
-        <v>118.305788635156</v>
+        <v>118.292412050625</v>
       </c>
       <c r="I22" t="n">
-        <v>-0.0940627427933384</v>
+        <v>-0.0940652362883882</v>
       </c>
       <c r="J22" t="n">
         <v>1</v>
@@ -9220,19 +9264,19 @@
         <v>2.36000000000008</v>
       </c>
       <c r="E23" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F23" t="n">
-        <v>152.112477383307</v>
+        <v>152.96998085039</v>
       </c>
       <c r="G23" t="n">
-        <v>-119.985788635156</v>
+        <v>-119.972412050625</v>
       </c>
       <c r="H23" t="n">
-        <v>124.705788635156</v>
+        <v>124.692412050625</v>
       </c>
       <c r="I23" t="n">
-        <v>0.054947542819875</v>
+        <v>0.0549489994159924</v>
       </c>
       <c r="J23" t="n">
         <v>1</v>
@@ -9249,22 +9293,22 @@
         <v>32</v>
       </c>
       <c r="D24" t="n">
-        <v>6.39999999999993</v>
+        <v>6.39999999999997</v>
       </c>
       <c r="E24" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F24" t="n">
-        <v>152.112477383307</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G24" t="n">
-        <v>-115.945788635156</v>
+        <v>-115.932412050625</v>
       </c>
       <c r="H24" t="n">
-        <v>128.745788635156</v>
+        <v>128.732412050625</v>
       </c>
       <c r="I24" t="n">
-        <v>0.149010285613213</v>
+        <v>0.14901423570438</v>
       </c>
       <c r="J24" t="n">
         <v>1</v>
@@ -9284,19 +9328,19 @@
         <v>3.71666666666678</v>
       </c>
       <c r="E25" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F25" t="n">
-        <v>152.112477383307</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G25" t="n">
-        <v>-118.629121968489</v>
+        <v>-118.615745383958</v>
       </c>
       <c r="H25" t="n">
-        <v>126.062455301822</v>
+        <v>126.049078717292</v>
       </c>
       <c r="I25" t="n">
-        <v>0.0865346189889269</v>
+        <v>0.0865369129220783</v>
       </c>
       <c r="J25" t="n">
         <v>1</v>
@@ -9313,22 +9357,22 @@
         <v>32</v>
       </c>
       <c r="D26" t="n">
-        <v>7.75666666666663</v>
+        <v>7.75666666666667</v>
       </c>
       <c r="E26" t="n">
-        <v>42.9500552506317</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F26" t="n">
-        <v>152.112477383307</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G26" t="n">
-        <v>-114.589121968489</v>
+        <v>-114.575745383958</v>
       </c>
       <c r="H26" t="n">
-        <v>130.102455301822</v>
+        <v>130.089078717292</v>
       </c>
       <c r="I26" t="n">
-        <v>0.180597361782265</v>
+        <v>0.180602149210466</v>
       </c>
       <c r="J26" t="n">
         <v>1</v>
@@ -9345,22 +9389,22 @@
         <v>32</v>
       </c>
       <c r="D27" t="n">
-        <v>1.35666666666669</v>
+        <v>1.3566666666667</v>
       </c>
       <c r="E27" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F27" t="n">
-        <v>152.112477383307</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G27" t="n">
-        <v>-120.989121968489</v>
+        <v>-120.975745383958</v>
       </c>
       <c r="H27" t="n">
-        <v>123.702455301822</v>
+        <v>123.689078717292</v>
       </c>
       <c r="I27" t="n">
-        <v>0.0315870761690519</v>
+        <v>0.0315879135060858</v>
       </c>
       <c r="J27" t="n">
         <v>1</v>
@@ -9377,22 +9421,22 @@
         <v>32</v>
       </c>
       <c r="D28" t="n">
-        <v>4.24333333333344</v>
+        <v>4.24333333333342</v>
       </c>
       <c r="E28" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F28" t="n">
-        <v>152.112477383307</v>
+        <v>152.96998085039</v>
       </c>
       <c r="G28" t="n">
-        <v>-118.102455301822</v>
+        <v>-118.089078717291</v>
       </c>
       <c r="H28" t="n">
-        <v>126.589121968489</v>
+        <v>126.575745383958</v>
       </c>
       <c r="I28" t="n">
-        <v>0.0987969237425142</v>
+        <v>0.0987995427352506</v>
       </c>
       <c r="J28" t="n">
         <v>1</v>
@@ -9409,22 +9453,22 @@
         <v>32</v>
       </c>
       <c r="D29" t="n">
-        <v>8.28333333333329</v>
+        <v>8.28333333333331</v>
       </c>
       <c r="E29" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F29" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G29" t="n">
-        <v>-114.062455301822</v>
+        <v>-114.049078717292</v>
       </c>
       <c r="H29" t="n">
-        <v>130.629121968489</v>
+        <v>130.615745383958</v>
       </c>
       <c r="I29" t="n">
-        <v>0.192859666535853</v>
+        <v>0.192864779023639</v>
       </c>
       <c r="J29" t="n">
         <v>1</v>
@@ -9441,22 +9485,22 @@
         <v>32</v>
       </c>
       <c r="D30" t="n">
-        <v>1.88333333333335</v>
+        <v>1.88333333333334</v>
       </c>
       <c r="E30" t="n">
-        <v>42.9500552506317</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F30" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G30" t="n">
-        <v>-120.462455301822</v>
+        <v>-120.449078717292</v>
       </c>
       <c r="H30" t="n">
-        <v>124.229121968489</v>
+        <v>124.215745383958</v>
       </c>
       <c r="I30" t="n">
-        <v>0.0438493809226393</v>
+        <v>0.0438505433192582</v>
       </c>
       <c r="J30" t="n">
         <v>1</v>
@@ -9473,22 +9517,22 @@
         <v>32</v>
       </c>
       <c r="D31" t="n">
-        <v>0.52666666666666</v>
+        <v>0.526666666666635</v>
       </c>
       <c r="E31" t="n">
-        <v>42.9500552506318</v>
+        <v>42.948916724282</v>
       </c>
       <c r="F31" t="n">
-        <v>152.112477383306</v>
+        <v>152.969980850391</v>
       </c>
       <c r="G31" t="n">
-        <v>-121.819121968489</v>
+        <v>-121.805745383958</v>
       </c>
       <c r="H31" t="n">
-        <v>122.872455301822</v>
+        <v>122.859078717292</v>
       </c>
       <c r="I31" t="n">
-        <v>0.0122623047535873</v>
+        <v>0.0122626298131723</v>
       </c>
       <c r="J31" t="n">
         <v>1</v>
@@ -9505,22 +9549,22 @@
         <v>33</v>
       </c>
       <c r="D32" t="n">
-        <v>-61.353977840109</v>
+        <v>-61.3140776089542</v>
       </c>
       <c r="E32" t="n">
-        <v>48.3422242811505</v>
+        <v>48.3117394362598</v>
       </c>
       <c r="F32" t="n">
-        <v>159.169822953763</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G32" t="n">
-        <v>-198.969512824457</v>
+        <v>-198.828678737239</v>
       </c>
       <c r="H32" t="n">
-        <v>76.261557144239</v>
+        <v>76.2005235193309</v>
       </c>
       <c r="I32" t="n">
-        <v>-1.26915918231822</v>
+        <v>-1.26913413436188</v>
       </c>
       <c r="J32" t="n">
         <v>1</v>
@@ -9537,22 +9581,22 @@
         <v>33</v>
       </c>
       <c r="D33" t="n">
-        <v>-72.2089987503088</v>
+        <v>-72.0761133493119</v>
       </c>
       <c r="E33" t="n">
-        <v>48.3422242811505</v>
+        <v>48.3117394362598</v>
       </c>
       <c r="F33" t="n">
-        <v>159.169822953763</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G33" t="n">
-        <v>-209.824533734657</v>
+        <v>-209.590714477597</v>
       </c>
       <c r="H33" t="n">
-        <v>65.4065362340392</v>
+        <v>65.4384877789733</v>
       </c>
       <c r="I33" t="n">
-        <v>-1.49370451658064</v>
+        <v>-1.49189646637347</v>
       </c>
       <c r="J33" t="n">
         <v>1</v>
@@ -9569,22 +9613,22 @@
         <v>33</v>
       </c>
       <c r="D34" t="n">
-        <v>-10.8550209101999</v>
+        <v>-10.7620357403577</v>
       </c>
       <c r="E34" t="n">
-        <v>48.3422242811505</v>
+        <v>48.3117394362598</v>
       </c>
       <c r="F34" t="n">
-        <v>159.16982295376</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G34" t="n">
-        <v>-148.470555894548</v>
+        <v>-148.276636868643</v>
       </c>
       <c r="H34" t="n">
-        <v>126.760514074148</v>
+        <v>126.752565387927</v>
       </c>
       <c r="I34" t="n">
-        <v>-0.224545334262422</v>
+        <v>-0.222762332011594</v>
       </c>
       <c r="J34" t="n">
         <v>1</v>
@@ -9601,22 +9645,22 @@
         <v>33</v>
       </c>
       <c r="D35" t="n">
-        <v>-57.7815902109837</v>
+        <v>-40.6047364478825</v>
       </c>
       <c r="E35" t="n">
-        <v>55.4559803093783</v>
+        <v>48.3117394362598</v>
       </c>
       <c r="F35" t="n">
-        <v>164.844207586982</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G35" t="n">
-        <v>-215.571150901421</v>
+        <v>-178.119337576168</v>
       </c>
       <c r="H35" t="n">
-        <v>100.007970479454</v>
+        <v>96.9098646804027</v>
       </c>
       <c r="I35" t="n">
-        <v>-1.04193614266002</v>
+        <v>-0.840473494055299</v>
       </c>
       <c r="J35" t="n">
         <v>1</v>
@@ -9633,22 +9677,22 @@
         <v>33</v>
       </c>
       <c r="D36" t="n">
-        <v>3.57238762912523</v>
+        <v>20.7093411610717</v>
       </c>
       <c r="E36" t="n">
-        <v>55.4559803093783</v>
+        <v>48.3117394362598</v>
       </c>
       <c r="F36" t="n">
-        <v>164.844207586981</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G36" t="n">
-        <v>-154.217173061312</v>
+        <v>-116.805259967213</v>
       </c>
       <c r="H36" t="n">
-        <v>161.361948319563</v>
+        <v>158.223942289357</v>
       </c>
       <c r="I36" t="n">
-        <v>0.0644184379970486</v>
+        <v>0.428660640306578</v>
       </c>
       <c r="J36" t="n">
         <v>1</v>
@@ -9665,22 +9709,22 @@
         <v>33</v>
       </c>
       <c r="D37" t="n">
-        <v>14.4274085393251</v>
+        <v>31.4713769014294</v>
       </c>
       <c r="E37" t="n">
-        <v>55.4559803093783</v>
+        <v>48.3117394362598</v>
       </c>
       <c r="F37" t="n">
-        <v>164.844207586981</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G37" t="n">
-        <v>-143.362152151112</v>
+        <v>-106.043224226856</v>
       </c>
       <c r="H37" t="n">
-        <v>172.216969229763</v>
+        <v>168.985978029714</v>
       </c>
       <c r="I37" t="n">
-        <v>0.260159652012955</v>
+        <v>0.651422972318172</v>
       </c>
       <c r="J37" t="n">
         <v>1</v>
@@ -9697,22 +9741,22 @@
         <v>33</v>
       </c>
       <c r="D38" t="n">
-        <v>-28.6419594336205</v>
+        <v>-27.9866089197955</v>
       </c>
       <c r="E38" t="n">
-        <v>48.3422242811504</v>
+        <v>48.3117394362598</v>
       </c>
       <c r="F38" t="n">
-        <v>159.169822953763</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G38" t="n">
-        <v>-166.257494417968</v>
+        <v>-165.501210048081</v>
       </c>
       <c r="H38" t="n">
-        <v>108.973575550727</v>
+        <v>109.52799220849</v>
       </c>
       <c r="I38" t="n">
-        <v>-0.592483276463316</v>
+        <v>-0.579292098491293</v>
       </c>
       <c r="J38" t="n">
         <v>1</v>
@@ -9729,22 +9773,22 @@
         <v>33</v>
       </c>
       <c r="D39" t="n">
-        <v>32.7120184064885</v>
+        <v>33.3274686891587</v>
       </c>
       <c r="E39" t="n">
-        <v>48.3422242811505</v>
+        <v>48.3117394362598</v>
       </c>
       <c r="F39" t="n">
-        <v>159.169822953761</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G39" t="n">
-        <v>-104.90351657786</v>
+        <v>-104.187132439126</v>
       </c>
       <c r="H39" t="n">
-        <v>170.327553390837</v>
+        <v>170.842069817444</v>
       </c>
       <c r="I39" t="n">
-        <v>0.676675905854905</v>
+        <v>0.689842035870585</v>
       </c>
       <c r="J39" t="n">
         <v>1</v>
@@ -9761,22 +9805,22 @@
         <v>33</v>
       </c>
       <c r="D40" t="n">
-        <v>43.5670393166884</v>
+        <v>44.0895044295164</v>
       </c>
       <c r="E40" t="n">
-        <v>48.3422242811505</v>
+        <v>48.3117394362598</v>
       </c>
       <c r="F40" t="n">
-        <v>159.16982295376</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G40" t="n">
-        <v>-94.0484956676598</v>
+        <v>-93.4250966987688</v>
       </c>
       <c r="H40" t="n">
-        <v>181.182574301036</v>
+        <v>181.604105557802</v>
       </c>
       <c r="I40" t="n">
-        <v>0.901221240117326</v>
+        <v>0.912604367882178</v>
       </c>
       <c r="J40" t="n">
         <v>1</v>
@@ -9793,22 +9837,22 @@
         <v>33</v>
       </c>
       <c r="D41" t="n">
-        <v>29.1396307773632</v>
+        <v>12.618127528087</v>
       </c>
       <c r="E41" t="n">
-        <v>55.4559803093783</v>
+        <v>48.3117394362598</v>
       </c>
       <c r="F41" t="n">
-        <v>164.844207586981</v>
+        <v>160.339008008648</v>
       </c>
       <c r="G41" t="n">
-        <v>-128.649929913074</v>
+        <v>-124.896473600198</v>
       </c>
       <c r="H41" t="n">
-        <v>186.929191467801</v>
+        <v>150.132728656372</v>
       </c>
       <c r="I41" t="n">
-        <v>0.525455155869553</v>
+        <v>0.261181395564007</v>
       </c>
       <c r="J41" t="n">
         <v>1</v>
@@ -9900,25 +9944,25 @@
         <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>-71.7366666666685</v>
+        <v>-71.7366666666684</v>
       </c>
       <c r="E2" t="n">
-        <v>21.6339256159408</v>
+        <v>21.5445960382291</v>
       </c>
       <c r="F2" t="n">
-        <v>175.328714368392</v>
+        <v>176.276267394501</v>
       </c>
       <c r="G2" t="n">
-        <v>-114.433094507242</v>
+        <v>-114.255206501281</v>
       </c>
       <c r="H2" t="n">
-        <v>-29.040238826095</v>
+        <v>-29.2181268320561</v>
       </c>
       <c r="I2" t="n">
-        <v>-3.31593386887722</v>
+        <v>-3.32968260529822</v>
       </c>
       <c r="J2" t="n">
-        <v>0.00111015725651823</v>
+        <v>0.00105880587902379</v>
       </c>
     </row>
     <row r="3">
@@ -9935,22 +9979,22 @@
         <v>-107.21</v>
       </c>
       <c r="E3" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382288</v>
       </c>
       <c r="F3" t="n">
-        <v>175.328714368372</v>
+        <v>176.276267394532</v>
       </c>
       <c r="G3" t="n">
-        <v>-149.906427840574</v>
+        <v>-149.728539834611</v>
       </c>
       <c r="H3" t="n">
-        <v>-64.5135721594263</v>
+        <v>-64.6914601653881</v>
       </c>
       <c r="I3" t="n">
-        <v>-4.95564244341317</v>
+        <v>-4.97618984406884</v>
       </c>
       <c r="J3" t="n">
-        <v>0.00000168961601207048</v>
+        <v>0.00000153331755227337</v>
       </c>
     </row>
     <row r="4">
@@ -9967,22 +10011,22 @@
         <v>-121.103333333333</v>
       </c>
       <c r="E4" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F4" t="n">
-        <v>175.328714368372</v>
+        <v>176.276267394532</v>
       </c>
       <c r="G4" t="n">
-        <v>-163.799761173907</v>
+        <v>-163.621873167945</v>
       </c>
       <c r="H4" t="n">
-        <v>-78.4069054927596</v>
+        <v>-78.5847934987219</v>
       </c>
       <c r="I4" t="n">
-        <v>-5.59784365922469</v>
+        <v>-5.6210537955062</v>
       </c>
       <c r="J4" t="n">
-        <v>0.000000082387851827143</v>
+        <v>0.000000073056848311268</v>
       </c>
     </row>
     <row r="5">
@@ -9996,25 +10040,25 @@
         <v>27</v>
       </c>
       <c r="D5" t="n">
-        <v>-85.1433333333335</v>
+        <v>-85.1433333333334</v>
       </c>
       <c r="E5" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F5" t="n">
-        <v>175.330398266293</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G5" t="n">
-        <v>-127.839758324169</v>
+        <v>-127.661873167945</v>
       </c>
       <c r="H5" t="n">
-        <v>-42.4469083424985</v>
+        <v>-42.6247934987219</v>
       </c>
       <c r="I5" t="n">
-        <v>-3.93563955265686</v>
+        <v>-3.95195775229459</v>
       </c>
       <c r="J5" t="n">
-        <v>0.000119478145328377</v>
+        <v>0.000112028278227113</v>
       </c>
     </row>
     <row r="6">
@@ -10031,22 +10075,22 @@
         <v>-122.223333333333</v>
       </c>
       <c r="E6" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382288</v>
       </c>
       <c r="F6" t="n">
-        <v>175.32871436837</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G6" t="n">
-        <v>-164.919761173907</v>
+        <v>-164.741873167945</v>
       </c>
       <c r="H6" t="n">
-        <v>-79.5269054927595</v>
+        <v>-79.7047934987217</v>
       </c>
       <c r="I6" t="n">
-        <v>-5.6496141986951</v>
+        <v>-5.67303898928808</v>
       </c>
       <c r="J6" t="n">
-        <v>0.000000063910935149058</v>
+        <v>0.0000000565627339115148</v>
       </c>
     </row>
     <row r="7">
@@ -10060,25 +10104,25 @@
         <v>27</v>
       </c>
       <c r="D7" t="n">
-        <v>-76.0866666666665</v>
+        <v>-76.0866666666664</v>
       </c>
       <c r="E7" t="n">
-        <v>21.633925615941</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F7" t="n">
-        <v>175.328714368376</v>
+        <v>176.276267394538</v>
       </c>
       <c r="G7" t="n">
-        <v>-118.78309450724</v>
+        <v>-118.605206501278</v>
       </c>
       <c r="H7" t="n">
-        <v>-33.3902388260926</v>
+        <v>-33.568126832055</v>
       </c>
       <c r="I7" t="n">
-        <v>-3.51700694628449</v>
+        <v>-3.53158938471895</v>
       </c>
       <c r="J7" t="n">
-        <v>0.000555743478415496</v>
+        <v>0.000527251117392954</v>
       </c>
     </row>
     <row r="8">
@@ -10095,22 +10139,22 @@
         <v>-76.2766666666667</v>
       </c>
       <c r="E8" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F8" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G8" t="n">
-        <v>-118.97309450724</v>
+        <v>-118.795206501278</v>
       </c>
       <c r="H8" t="n">
-        <v>-33.580238826093</v>
+        <v>-33.7581268320552</v>
       </c>
       <c r="I8" t="n">
-        <v>-3.52578944851611</v>
+        <v>-3.54040830152124</v>
       </c>
       <c r="J8" t="n">
-        <v>0.00053882382080851</v>
+        <v>0.000511078352599034</v>
       </c>
     </row>
     <row r="9">
@@ -10124,25 +10168,25 @@
         <v>27</v>
       </c>
       <c r="D9" t="n">
-        <v>-81.5</v>
+        <v>-81.4999999999999</v>
       </c>
       <c r="E9" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F9" t="n">
-        <v>175.32871436837</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G9" t="n">
-        <v>-124.196427840574</v>
+        <v>-124.018539834611</v>
       </c>
       <c r="H9" t="n">
-        <v>-38.8035721594263</v>
+        <v>-38.9814601653884</v>
       </c>
       <c r="I9" t="n">
-        <v>-3.7672312203915</v>
+        <v>-3.78285115466479</v>
       </c>
       <c r="J9" t="n">
-        <v>0.000225192424756205</v>
+        <v>0.000212177496497988</v>
       </c>
     </row>
     <row r="10">
@@ -10159,22 +10203,22 @@
         <v>-111.643333333333</v>
       </c>
       <c r="E10" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F10" t="n">
-        <v>175.330398266296</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G10" t="n">
-        <v>-154.339758324168</v>
+        <v>-154.161873167945</v>
       </c>
       <c r="H10" t="n">
-        <v>-68.9469083424983</v>
+        <v>-69.1247934987217</v>
       </c>
       <c r="I10" t="n">
-        <v>-5.16056749548354</v>
+        <v>-5.18196456945553</v>
       </c>
       <c r="J10" t="n">
-        <v>0.00000066185551756281</v>
+        <v>0.000000596334691284294</v>
       </c>
     </row>
     <row r="11">
@@ -10188,25 +10232,25 @@
         <v>27</v>
       </c>
       <c r="D11" t="n">
-        <v>-89.1533333333334</v>
+        <v>-89.1533333333333</v>
       </c>
       <c r="E11" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F11" t="n">
-        <v>175.32871436837</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G11" t="n">
-        <v>-131.849761173907</v>
+        <v>-131.671873167945</v>
       </c>
       <c r="H11" t="n">
-        <v>-46.4569054927596</v>
+        <v>-46.6347934987218</v>
       </c>
       <c r="I11" t="n">
-        <v>-4.12099657343931</v>
+        <v>-4.13808331217442</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0000580920250110722</v>
+        <v>0.0000541692859301372</v>
       </c>
     </row>
     <row r="12">
@@ -10220,25 +10264,25 @@
         <v>31</v>
       </c>
       <c r="D12" t="n">
-        <v>-67.9066666666665</v>
+        <v>-67.9066666666666</v>
       </c>
       <c r="E12" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F12" t="n">
-        <v>175.328714368374</v>
+        <v>176.276267394525</v>
       </c>
       <c r="G12" t="n">
-        <v>-110.60309450724</v>
+        <v>-110.425206501278</v>
       </c>
       <c r="H12" t="n">
-        <v>-25.2102388260928</v>
+        <v>-25.3881268320551</v>
       </c>
       <c r="I12" t="n">
-        <v>-3.13889711336669</v>
+        <v>-3.15191180870475</v>
       </c>
       <c r="J12" t="n">
-        <v>0.00199012947709015</v>
+        <v>0.00190650082600691</v>
       </c>
     </row>
     <row r="13">
@@ -10252,25 +10296,25 @@
         <v>31</v>
       </c>
       <c r="D13" t="n">
-        <v>-61.7633333333334</v>
+        <v>-61.7633333333333</v>
       </c>
       <c r="E13" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F13" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G13" t="n">
-        <v>-104.459761173907</v>
+        <v>-104.281873167945</v>
       </c>
       <c r="H13" t="n">
-        <v>-19.0669054927596</v>
+        <v>-19.2447934987218</v>
       </c>
       <c r="I13" t="n">
-        <v>-2.85492954121203</v>
+        <v>-2.8667668320975</v>
       </c>
       <c r="J13" t="n">
-        <v>0.00482405715612643</v>
+        <v>0.00465232614469612</v>
       </c>
     </row>
     <row r="14">
@@ -10287,22 +10331,22 @@
         <v>-115.193333333333</v>
       </c>
       <c r="E14" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F14" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G14" t="n">
-        <v>-157.889761173907</v>
+        <v>-157.711873167945</v>
       </c>
       <c r="H14" t="n">
-        <v>-72.4969054927597</v>
+        <v>-72.6747934987219</v>
       </c>
       <c r="I14" t="n">
-        <v>-5.32466161612636</v>
+        <v>-5.34673906760351</v>
       </c>
       <c r="J14" t="n">
-        <v>0.000000306816249806462</v>
+        <v>0.000000274817123436198</v>
       </c>
     </row>
     <row r="15">
@@ -10319,22 +10363,22 @@
         <v>-134.216666666667</v>
       </c>
       <c r="E15" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F15" t="n">
-        <v>175.330398266296</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G15" t="n">
-        <v>-176.913091657502</v>
+        <v>-176.735206501278</v>
       </c>
       <c r="H15" t="n">
-        <v>-91.5202416758317</v>
+        <v>-91.6981268320551</v>
       </c>
       <c r="I15" t="n">
-        <v>-6.20399039219075</v>
+        <v>-6.22971377270257</v>
       </c>
       <c r="J15" t="n">
-        <v>0.00000000384839253840501</v>
+        <v>0.00000000333384861835068</v>
       </c>
     </row>
     <row r="16">
@@ -10351,22 +10395,22 @@
         <v>-90.6066666666667</v>
       </c>
       <c r="E16" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F16" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G16" t="n">
-        <v>-133.30309450724</v>
+        <v>-133.125206501278</v>
       </c>
       <c r="H16" t="n">
-        <v>-47.9102388260929</v>
+        <v>-48.0881268320552</v>
       </c>
       <c r="I16" t="n">
-        <v>-4.18817501156162</v>
+        <v>-4.20554028981998</v>
       </c>
       <c r="J16" t="n">
-        <v>0.0000444648145343288</v>
+        <v>0.0000413773177673957</v>
       </c>
     </row>
     <row r="17">
@@ -10380,25 +10424,25 @@
         <v>31</v>
       </c>
       <c r="D17" t="n">
-        <v>-79.4666666666667</v>
+        <v>-79.4666666666668</v>
       </c>
       <c r="E17" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F17" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G17" t="n">
-        <v>-122.16309450724</v>
+        <v>-121.985206501278</v>
       </c>
       <c r="H17" t="n">
-        <v>-36.770238826093</v>
+        <v>-36.9481268320553</v>
       </c>
       <c r="I17" t="n">
-        <v>-3.67324303861486</v>
+        <v>-3.68847327309647</v>
       </c>
       <c r="J17" t="n">
-        <v>0.000317888058032863</v>
+        <v>0.000300306531834086</v>
       </c>
     </row>
     <row r="18">
@@ -10415,22 +10459,22 @@
         <v>-58.37</v>
       </c>
       <c r="E18" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382288</v>
       </c>
       <c r="F18" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G18" t="n">
-        <v>-101.066427840574</v>
+        <v>-100.888539834612</v>
       </c>
       <c r="H18" t="n">
-        <v>-15.6735721594263</v>
+        <v>-15.8514601653885</v>
       </c>
       <c r="I18" t="n">
-        <v>-2.69807713293561</v>
+        <v>-2.70926407236544</v>
       </c>
       <c r="J18" t="n">
-        <v>0.00765563760177036</v>
+        <v>0.00740870990658255</v>
       </c>
     </row>
     <row r="19">
@@ -10447,22 +10491,22 @@
         <v>-63.47</v>
       </c>
       <c r="E19" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F19" t="n">
-        <v>175.328714368374</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G19" t="n">
-        <v>-106.166427840574</v>
+        <v>-105.988539834612</v>
       </c>
       <c r="H19" t="n">
-        <v>-20.7735721594263</v>
+        <v>-20.9514601653885</v>
       </c>
       <c r="I19" t="n">
-        <v>-2.9338179823098</v>
+        <v>-2.94598236547944</v>
       </c>
       <c r="J19" t="n">
-        <v>0.00379612709966472</v>
+        <v>0.0036543934932541</v>
       </c>
     </row>
     <row r="20">
@@ -10479,22 +10523,22 @@
         <v>-77.09</v>
       </c>
       <c r="E20" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F20" t="n">
-        <v>175.330398266293</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G20" t="n">
-        <v>-119.786424990835</v>
+        <v>-119.608539834611</v>
       </c>
       <c r="H20" t="n">
-        <v>-34.393575009165</v>
+        <v>-34.5714601653886</v>
       </c>
       <c r="I20" t="n">
-        <v>-3.56338472122675</v>
+        <v>-3.57815945414858</v>
       </c>
       <c r="J20" t="n">
-        <v>0.000471718516563954</v>
+        <v>0.00044697561903417</v>
       </c>
     </row>
     <row r="21">
@@ -10511,22 +10555,22 @@
         <v>-51.1433333333333</v>
       </c>
       <c r="E21" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F21" t="n">
-        <v>175.328714368372</v>
+        <v>176.276267394532</v>
       </c>
       <c r="G21" t="n">
-        <v>-93.8397611739071</v>
+        <v>-93.6618731679448</v>
       </c>
       <c r="H21" t="n">
-        <v>-8.44690549275963</v>
+        <v>-8.62479349872185</v>
       </c>
       <c r="I21" t="n">
-        <v>-2.36403389016224</v>
+        <v>-2.3738357982013</v>
       </c>
       <c r="J21" t="n">
-        <v>0.0191714422654657</v>
+        <v>0.018679954061264</v>
       </c>
     </row>
     <row r="22">
@@ -10540,25 +10584,25 @@
         <v>32</v>
       </c>
       <c r="D22" t="n">
-        <v>-43.7466666666665</v>
+        <v>-43.7466666666666</v>
       </c>
       <c r="E22" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F22" t="n">
-        <v>175.328714368372</v>
+        <v>176.276267394527</v>
       </c>
       <c r="G22" t="n">
-        <v>-86.4430945072403</v>
+        <v>-86.265206501278</v>
       </c>
       <c r="H22" t="n">
-        <v>-1.05023882609281</v>
+        <v>-1.22812683205516</v>
       </c>
       <c r="I22" t="n">
-        <v>-2.0221326190764</v>
+        <v>-2.0305169142667</v>
       </c>
       <c r="J22" t="n">
-        <v>0.0446826202247278</v>
+        <v>0.0438066350498603</v>
       </c>
     </row>
     <row r="23">
@@ -10575,22 +10619,22 @@
         <v>-32.2233333333334</v>
       </c>
       <c r="E23" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F23" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G23" t="n">
-        <v>-74.9197611739071</v>
+        <v>-74.7418731679448</v>
       </c>
       <c r="H23" t="n">
-        <v>10.4730945072403</v>
+        <v>10.2952065012781</v>
       </c>
       <c r="I23" t="n">
-        <v>-1.48948156267995</v>
+        <v>-1.49565734609998</v>
       </c>
       <c r="J23" t="n">
-        <v>0.138157244805313</v>
+        <v>0.136531125187442</v>
       </c>
     </row>
     <row r="24">
@@ -10607,22 +10651,22 @@
         <v>-47.23</v>
       </c>
       <c r="E24" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F24" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G24" t="n">
-        <v>-89.9264278405737</v>
+        <v>-89.7485398346115</v>
       </c>
       <c r="H24" t="n">
-        <v>-4.53357215942627</v>
+        <v>-4.71146016538854</v>
       </c>
       <c r="I24" t="n">
-        <v>-2.18314515998884</v>
+        <v>-2.19219705564194</v>
       </c>
       <c r="J24" t="n">
-        <v>0.0303539940787899</v>
+        <v>0.0296755936463832</v>
       </c>
     </row>
     <row r="25">
@@ -10639,22 +10683,22 @@
         <v>-52.7</v>
       </c>
       <c r="E25" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F25" t="n">
-        <v>175.330398266296</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G25" t="n">
-        <v>-95.396424990835</v>
+        <v>-95.2185398346115</v>
       </c>
       <c r="H25" t="n">
-        <v>-10.003575009165</v>
+        <v>-10.1814601653886</v>
       </c>
       <c r="I25" t="n">
-        <v>-2.43598877686665</v>
+        <v>-2.4460890288446</v>
       </c>
       <c r="J25" t="n">
-        <v>0.0158516115915486</v>
+        <v>0.0154235857868347</v>
       </c>
     </row>
     <row r="26">
@@ -10671,22 +10715,22 @@
         <v>-39.7933333333333</v>
       </c>
       <c r="E26" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F26" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G26" t="n">
-        <v>-82.489761173907</v>
+        <v>-82.3118731679448</v>
       </c>
       <c r="H26" t="n">
-        <v>2.90309450724035</v>
+        <v>2.72520650127819</v>
       </c>
       <c r="I26" t="n">
-        <v>-1.83939494106478</v>
+        <v>-1.84702155764369</v>
       </c>
       <c r="J26" t="n">
-        <v>0.0675482846527321</v>
+        <v>0.0664202826001771</v>
       </c>
     </row>
     <row r="27">
@@ -10703,22 +10747,22 @@
         <v>-36.78</v>
       </c>
       <c r="E27" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F27" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G27" t="n">
-        <v>-79.4764278405737</v>
+        <v>-79.2985398346115</v>
       </c>
       <c r="H27" t="n">
-        <v>5.91642784057373</v>
+        <v>5.73853983461145</v>
       </c>
       <c r="I27" t="n">
-        <v>-1.70010753725152</v>
+        <v>-1.70715663151621</v>
       </c>
       <c r="J27" t="n">
-        <v>0.0908839039451707</v>
+        <v>0.0895536716781867</v>
       </c>
     </row>
     <row r="28">
@@ -10735,22 +10779,22 @@
         <v>-29.2966666666667</v>
       </c>
       <c r="E28" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F28" t="n">
-        <v>175.328714368372</v>
+        <v>176.276267394532</v>
       </c>
       <c r="G28" t="n">
-        <v>-71.9930945072404</v>
+        <v>-71.8152065012781</v>
       </c>
       <c r="H28" t="n">
-        <v>13.399761173907</v>
+        <v>13.2218731679448</v>
       </c>
       <c r="I28" t="n">
-        <v>-1.35420021251619</v>
+        <v>-1.35981508377705</v>
       </c>
       <c r="J28" t="n">
-        <v>0.177415291629468</v>
+        <v>0.175625150440316</v>
       </c>
     </row>
     <row r="29">
@@ -10764,25 +10808,25 @@
         <v>32</v>
       </c>
       <c r="D29" t="n">
-        <v>-37.9033333333333</v>
+        <v>-37.9033333333334</v>
       </c>
       <c r="E29" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F29" t="n">
-        <v>175.328714368374</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G29" t="n">
-        <v>-80.5997611739071</v>
+        <v>-80.4218731679448</v>
       </c>
       <c r="H29" t="n">
-        <v>4.79309450724042</v>
+        <v>4.61520650127809</v>
       </c>
       <c r="I29" t="n">
-        <v>-1.75203215570845</v>
+        <v>-1.75929654313674</v>
       </c>
       <c r="J29" t="n">
-        <v>0.0815165821073071</v>
+        <v>0.0802620379819752</v>
       </c>
     </row>
     <row r="30">
@@ -10799,22 +10843,22 @@
         <v>-42.0166666666667</v>
       </c>
       <c r="E30" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F30" t="n">
-        <v>175.330398266296</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G30" t="n">
-        <v>-84.7130916575018</v>
+        <v>-84.5352065012781</v>
       </c>
       <c r="H30" t="n">
-        <v>0.679758324168418</v>
+        <v>0.501873167944723</v>
       </c>
       <c r="I30" t="n">
-        <v>-1.942165625073</v>
+        <v>-1.95021835601431</v>
       </c>
       <c r="J30" t="n">
-        <v>0.0537194269555285</v>
+        <v>0.0527360808103929</v>
       </c>
     </row>
     <row r="31">
@@ -10831,22 +10875,22 @@
         <v>-28.5833333333333</v>
       </c>
       <c r="E31" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F31" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G31" t="n">
-        <v>-71.2797611739071</v>
+        <v>-71.1018731679448</v>
       </c>
       <c r="H31" t="n">
-        <v>14.1130945072404</v>
+        <v>13.9352065012781</v>
       </c>
       <c r="I31" t="n">
-        <v>-1.32122730940111</v>
+        <v>-1.32670546630882</v>
       </c>
       <c r="J31" t="n">
-        <v>0.188147226172773</v>
+        <v>0.186322236165336</v>
       </c>
     </row>
     <row r="32">
@@ -10863,22 +10907,22 @@
         <v>-134.172884283333</v>
       </c>
       <c r="E32" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382288</v>
       </c>
       <c r="F32" t="n">
-        <v>175.328714368379</v>
+        <v>176.276267394527</v>
       </c>
       <c r="G32" t="n">
-        <v>-176.869312123907</v>
+        <v>-176.691424117945</v>
       </c>
       <c r="H32" t="n">
-        <v>-91.4764564427597</v>
+        <v>-91.6543444487217</v>
       </c>
       <c r="I32" t="n">
-        <v>-6.20196660861533</v>
+        <v>-6.22768159798665</v>
       </c>
       <c r="J32" t="n">
-        <v>0.00000000388925974776564</v>
+        <v>0.00000000336946646177533</v>
       </c>
     </row>
     <row r="33">
@@ -10895,22 +10939,22 @@
         <v>-71.0008162</v>
       </c>
       <c r="E33" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F33" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G33" t="n">
-        <v>-113.697244040574</v>
+        <v>-113.519356034612</v>
       </c>
       <c r="H33" t="n">
-        <v>-28.3043883594263</v>
+        <v>-28.4822763653884</v>
       </c>
       <c r="I33" t="n">
-        <v>-3.28192014063704</v>
+        <v>-3.29552784716948</v>
       </c>
       <c r="J33" t="n">
-        <v>0.00124422743155432</v>
+        <v>0.00118770323847704</v>
       </c>
     </row>
     <row r="34">
@@ -10924,25 +10968,25 @@
         <v>33</v>
       </c>
       <c r="D34" t="n">
-        <v>-79.5745103966667</v>
+        <v>-79.5745103966666</v>
       </c>
       <c r="E34" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F34" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G34" t="n">
-        <v>-122.27093823724</v>
+        <v>-122.093050231278</v>
       </c>
       <c r="H34" t="n">
-        <v>-36.878082556093</v>
+        <v>-37.0559705620551</v>
       </c>
       <c r="I34" t="n">
-        <v>-3.67822797440111</v>
+        <v>-3.6934788777413</v>
       </c>
       <c r="J34" t="n">
-        <v>0.000312179390112868</v>
+        <v>0.000294872746609905</v>
       </c>
     </row>
     <row r="35">
@@ -10959,22 +11003,22 @@
         <v>-94.8536093833333</v>
       </c>
       <c r="E35" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F35" t="n">
-        <v>175.330398266296</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G35" t="n">
-        <v>-137.550034374168</v>
+        <v>-137.372149217945</v>
       </c>
       <c r="H35" t="n">
-        <v>-52.1571843924984</v>
+        <v>-52.3350695487218</v>
       </c>
       <c r="I35" t="n">
-        <v>-4.38448440043821</v>
+        <v>-4.4026636292008</v>
       </c>
       <c r="J35" t="n">
-        <v>0.0000199973328081164</v>
+        <v>0.0000184950831484385</v>
       </c>
     </row>
     <row r="36">
@@ -10988,25 +11032,25 @@
         <v>33</v>
       </c>
       <c r="D36" t="n">
-        <v>-87.9172808433333</v>
+        <v>-87.9172808433332</v>
       </c>
       <c r="E36" t="n">
-        <v>21.6339256159409</v>
+        <v>21.5445960382287</v>
       </c>
       <c r="F36" t="n">
-        <v>175.328714368372</v>
+        <v>176.27626739453</v>
       </c>
       <c r="G36" t="n">
-        <v>-130.613708683907</v>
+        <v>-130.435820677945</v>
       </c>
       <c r="H36" t="n">
-        <v>-45.2208530027596</v>
+        <v>-45.3987410087217</v>
       </c>
       <c r="I36" t="n">
-        <v>-4.06386165895623</v>
+        <v>-4.08071150126616</v>
       </c>
       <c r="J36" t="n">
-        <v>0.0000727406442716959</v>
+        <v>0.0000679458280421708</v>
       </c>
     </row>
     <row r="37">
@@ -11020,25 +11064,25 @@
         <v>33</v>
       </c>
       <c r="D37" t="n">
-        <v>-87.6768890728001</v>
+        <v>-87.5492549207071</v>
       </c>
       <c r="E37" t="n">
-        <v>26.7237429781913</v>
+        <v>26.6247437214771</v>
       </c>
       <c r="F37" t="n">
-        <v>175.585158321594</v>
+        <v>176.326806165861</v>
       </c>
       <c r="G37" t="n">
-        <v>-140.417977445053</v>
+        <v>-140.093428031031</v>
       </c>
       <c r="H37" t="n">
-        <v>-34.9358007005477</v>
+        <v>-35.0050818103833</v>
       </c>
       <c r="I37" t="n">
-        <v>-3.28086111082386</v>
+        <v>-3.28826657775807</v>
       </c>
       <c r="J37" t="n">
-        <v>0.00124830487104552</v>
+        <v>0.0012168647740361</v>
       </c>
     </row>
     <row r="38">
@@ -11052,25 +11096,25 @@
         <v>33</v>
       </c>
       <c r="D38" t="n">
-        <v>-85.8587988295757</v>
+        <v>-85.6912644463279</v>
       </c>
       <c r="E38" t="n">
-        <v>26.7237429781913</v>
+        <v>26.6247437214771</v>
       </c>
       <c r="F38" t="n">
-        <v>175.585158321594</v>
+        <v>176.326806165861</v>
       </c>
       <c r="G38" t="n">
-        <v>-138.599887201828</v>
+        <v>-138.235437556652</v>
       </c>
       <c r="H38" t="n">
-        <v>-33.1177104573233</v>
+        <v>-33.1470913360042</v>
       </c>
       <c r="I38" t="n">
-        <v>-3.21282834143567</v>
+        <v>-3.21848222626099</v>
       </c>
       <c r="J38" t="n">
-        <v>0.00156382270854653</v>
+        <v>0.00153392864792537</v>
       </c>
     </row>
     <row r="39">
@@ -11084,25 +11128,25 @@
         <v>33</v>
       </c>
       <c r="D39" t="n">
-        <v>-105.287513936442</v>
+        <v>-105.026994383352</v>
       </c>
       <c r="E39" t="n">
-        <v>26.7237429781914</v>
+        <v>26.6247437214771</v>
       </c>
       <c r="F39" t="n">
-        <v>175.585158321594</v>
+        <v>176.326806165861</v>
       </c>
       <c r="G39" t="n">
-        <v>-158.028602308695</v>
+        <v>-157.571167493676</v>
       </c>
       <c r="H39" t="n">
-        <v>-52.5464255641898</v>
+        <v>-52.4828212730286</v>
       </c>
       <c r="I39" t="n">
-        <v>-3.93984907063225</v>
+        <v>-3.94471381516552</v>
       </c>
       <c r="J39" t="n">
-        <v>0.000117510263373635</v>
+        <v>0.000115172816972565</v>
       </c>
     </row>
     <row r="40">
@@ -11116,25 +11160,25 @@
         <v>33</v>
       </c>
       <c r="D40" t="n">
-        <v>-106.139204383784</v>
+        <v>-88.8347164685895</v>
       </c>
       <c r="E40" t="n">
-        <v>38.1123804345718</v>
+        <v>26.6247437214771</v>
       </c>
       <c r="F40" t="n">
-        <v>175.596207610023</v>
+        <v>176.326806165861</v>
       </c>
       <c r="G40" t="n">
-        <v>-181.356495184283</v>
+        <v>-141.378889578913</v>
       </c>
       <c r="H40" t="n">
-        <v>-30.9219135832841</v>
+        <v>-36.2905433582659</v>
       </c>
       <c r="I40" t="n">
-        <v>-2.78490094750169</v>
+        <v>-3.33654728841316</v>
       </c>
       <c r="J40" t="n">
-        <v>0.00594209680427218</v>
+        <v>0.00103447088621667</v>
       </c>
     </row>
     <row r="41">
@@ -11148,25 +11192,25 @@
         <v>33</v>
       </c>
       <c r="D41" t="n">
-        <v>-70.0632450664205</v>
+        <v>-69.2802604005025</v>
       </c>
       <c r="E41" t="n">
-        <v>26.7237429781913</v>
+        <v>26.6247437214771</v>
       </c>
       <c r="F41" t="n">
-        <v>175.585158321594</v>
+        <v>176.326806165858</v>
       </c>
       <c r="G41" t="n">
-        <v>-122.804333438673</v>
+        <v>-121.824433510826</v>
       </c>
       <c r="H41" t="n">
-        <v>-17.3221566941681</v>
+        <v>-16.7360872901788</v>
       </c>
       <c r="I41" t="n">
-        <v>-2.6217601749724</v>
+        <v>-2.60210055447846</v>
       </c>
       <c r="J41" t="n">
-        <v>0.0095156819419956</v>
+        <v>0.010053420055365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>